<commit_message>
Added RegEx pdf flow, added populate queue flow, updated config, added input file samples
</commit_message>
<xml_diff>
--- a/RegEx Document Processing Demo/Data/Config.xlsx
+++ b/RegEx Document Processing Demo/Data/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uipath-my.sharepoint.com/personal/alexandra_veizu_uipath_com/Documents/Documents/Projects/REFrameworkNET5/StudioTemplates/REFramework/contentFiles/any/any/pt2/VisualBasic/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci\Documents\UiPath\REPO\RegEx Document Processing Demo\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8C54E24-BA5C-4BF9-8DAB-2778512EC11B}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D22AE03-444F-427A-BA18-5936DBF4EAE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
   <si>
     <t>Name</t>
   </si>
@@ -85,9 +85,6 @@
   </si>
   <si>
     <t>logF_BusinessProcessName</t>
-  </si>
-  <si>
-    <t>Framework</t>
   </si>
   <si>
     <t>Orchestrator queue Name. The value must match with the queue name defined on Orchestrator.</t>
@@ -159,14 +156,77 @@
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
   </si>
   <si>
-    <t>ProcessABCQueue</t>
+    <t>RegEx Document Processing Demo</t>
+  </si>
+  <si>
+    <t>RegEx_Document_Processing_Demo</t>
+  </si>
+  <si>
+    <t>InputFolder</t>
+  </si>
+  <si>
+    <t>OutputFolder</t>
+  </si>
+  <si>
+    <t>TempFolder</t>
+  </si>
+  <si>
+    <t>Data\Input</t>
+  </si>
+  <si>
+    <t>Data\Output</t>
+  </si>
+  <si>
+    <t>Data\Temp</t>
+  </si>
+  <si>
+    <t>RegEx_PDF_Date</t>
+  </si>
+  <si>
+    <t>RegEx_PDF_Number</t>
+  </si>
+  <si>
+    <t>RegEx_PDF_Vendor</t>
+  </si>
+  <si>
+    <t>RegEx_PDF_TotalAmount</t>
+  </si>
+  <si>
+    <t>(?&lt;=INVOICE\\r\\n# )\d{5,10}(?=\\r)</t>
+  </si>
+  <si>
+    <t>RegEx_PDF_Lines</t>
+  </si>
+  <si>
+    <t>RegEx_PDF_LineGroup</t>
+  </si>
+  <si>
+    <t>(?&lt;=Amount\\r\\n\\r\\n).*(?=\\r\\n\\r\\nSubtotal)</t>
+  </si>
+  <si>
+    <t>^(.*?),.*?\s+(\d+)\s+\$?(\d{1,3}(?:,\d{3})*\.\d{2})\s+\$?(\d{1,3}(?:,\d{3})*\.\d{2})</t>
+  </si>
+  <si>
+    <t>(?&lt;=Date: )[A-Za-z]{3}\s+\d{1,2}\s+\d{4}(?=\\r\\n)</t>
+  </si>
+  <si>
+    <t>(?&lt;=Balance Due: )\$?(\d{1,3}(?:,\d{3})*\.\d{2})(?=\\r\\n\\r\\nItem Quantity)</t>
+  </si>
+  <si>
+    <t>^(.*?)\s+(?=INVOICE)</t>
+  </si>
+  <si>
+    <t>RegEx_PDF_Order</t>
+  </si>
+  <si>
+    <t>(?&lt;=Order ID : ).*</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -190,6 +250,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -211,19 +277,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normalny" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -239,9 +306,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Motyw pakietu Office">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Pakiet Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -279,7 +346,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Pakiet Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -385,7 +452,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Pakiet Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -535,13 +602,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z998"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:Z999"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5546875" customWidth="1"/>
-    <col min="2" max="2" width="43" customWidth="1"/>
-    <col min="3" max="3" width="81.44140625" customWidth="1"/>
-    <col min="4" max="26" width="8.6640625" customWidth="1"/>
+    <col min="1" max="1" width="43.5703125" customWidth="1"/>
+    <col min="2" max="2" width="74.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="88.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -580,63 +647,133 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>44</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="43.2">
+    <row r="3" spans="1:26" ht="45">
       <c r="A3" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="28.8">
+    <row r="5" spans="1:26" ht="30">
       <c r="A5" t="s">
         <v>20</v>
       </c>
-      <c r="B5" t="s">
-        <v>21</v>
+      <c r="B5" s="5" t="s">
+        <v>43</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+    </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" ht="14.25" customHeight="1"/>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B17" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="19" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="20" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="21" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="22" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="23" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="24" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="25" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="26" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="27" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="29" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="30" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="31" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="32" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>
@@ -1603,6 +1740,7 @@
     <row r="996" ht="14.25" customHeight="1"/>
     <row r="997" ht="14.25" customHeight="1"/>
     <row r="998" ht="14.25" customHeight="1"/>
+    <row r="999" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1613,12 +1751,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.44140625" customWidth="1"/>
-    <col min="4" max="26" width="8.6640625" customWidth="1"/>
+    <col min="3" max="3" width="75.42578125" customWidth="1"/>
+    <col min="4" max="26" width="8.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -1655,7 +1793,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="28.8">
+    <row r="2" spans="1:26" ht="30">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1663,18 +1801,18 @@
         <v>0</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="43.2">
+    <row r="3" spans="1:26" ht="45">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B3">
         <v>0</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1698,7 +1836,7 @@
         <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
@@ -1720,7 +1858,7 @@
         <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
@@ -1731,7 +1869,7 @@
         <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
@@ -1742,53 +1880,53 @@
         <v>19</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14">
         <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B15">
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="28.8">
+    <row r="17" spans="1:3" ht="45">
       <c r="A17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B17" t="b">
         <v>0</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1"/>
@@ -2771,12 +2909,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.88671875" customWidth="1"/>
-    <col min="2" max="2" width="30.109375" customWidth="1"/>
-    <col min="3" max="3" width="60.33203125" customWidth="1"/>
-    <col min="4" max="26" width="65.44140625" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" customWidth="1"/>
+    <col min="3" max="3" width="60.28515625" customWidth="1"/>
+    <col min="4" max="26" width="65.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -2787,7 +2925,7 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
Added more pdfs to the input folder, changed regex_pdf flow logic
</commit_message>
<xml_diff>
--- a/RegEx Document Processing Demo/Data/Config.xlsx
+++ b/RegEx Document Processing Demo/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci\Documents\UiPath\REPO\RegEx Document Processing Demo\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C233F3A-A8C1-4355-96B4-F1CA959DE27B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF78F62-8BDC-45D4-ADDF-4AC9CD388057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
   <si>
     <t>Name</t>
   </si>
@@ -180,52 +180,46 @@
     <t>Data\Temp</t>
   </si>
   <si>
-    <t>RegEx_PDF_Date</t>
-  </si>
-  <si>
-    <t>RegEx_PDF_Number</t>
-  </si>
-  <si>
-    <t>RegEx_PDF_Vendor</t>
-  </si>
-  <si>
-    <t>RegEx_PDF_Lines</t>
-  </si>
-  <si>
-    <t>RegEx_PDF_LineGroup</t>
-  </si>
-  <si>
     <t>^(.*?)\s+(?=INVOICE)</t>
   </si>
   <si>
-    <t>RegEx_PDF_Order</t>
-  </si>
-  <si>
     <t>(?&lt;=Order ID : ).*</t>
   </si>
   <si>
     <t>(?&lt;=INVOICE\r\n# )\d{5,10}(?=\r)</t>
   </si>
   <si>
-    <t>(?&lt;=Amount\r\n\r\n).*(?=\r\n\r\nSubtotal)</t>
-  </si>
-  <si>
-    <t>RegEx_PDF_Amount</t>
-  </si>
-  <si>
     <t>[A-Za-z]{3}\s+\d{1,2}\s+\d{4}</t>
   </si>
   <si>
     <t>\$?\d{1,3}(?:,\d{3})*\.\d{2}</t>
   </si>
   <si>
-    <t>(?&lt;=Rate Amount\r\n\r\n)(.*?),.*?\s+(\d+)\s+\$?(\d{1,3}(?:,\d{3})*\.\d{2})\s+\$?(\d{1,3}(?:,\d{3})*\.\d{2})</t>
-  </si>
-  <si>
     <t>ExtractionSuccessThreshold</t>
   </si>
   <si>
     <t>0.9</t>
+  </si>
+  <si>
+    <t>RegEx_PDF_Header_Date</t>
+  </si>
+  <si>
+    <t>RegEx_PDF_Header_Number</t>
+  </si>
+  <si>
+    <t>RegEx_PDF_Header_Vendor</t>
+  </si>
+  <si>
+    <t>RegEx_PDF_Header_Amount</t>
+  </si>
+  <si>
+    <t>RegEx_PDF_Body_LineGroup</t>
+  </si>
+  <si>
+    <t>RegEx_PDF_Footer_Order</t>
+  </si>
+  <si>
+    <t>(?&lt;=Rate Amount\r\n\r\n)(.*).*?\s+(\d+)\s+\$?(\d{1,3}(?:,\d{3})*\.\d{2})\s+\$?(\d{1,3}(?:,\d{3})*\.\d{2})</t>
   </si>
 </sst>
 </file>
@@ -608,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z999"/>
+  <dimension ref="A1:Z998"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -711,26 +705,26 @@
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="B13" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
@@ -738,42 +732,35 @@
         <v>61</v>
       </c>
       <c r="B14" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B15" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="B16" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A17" t="s">
+    <row r="17" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="18" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" t="s">
         <v>57</v>
       </c>
-      <c r="B17" t="s">
-        <v>58</v>
-      </c>
     </row>
-    <row r="18" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="19" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A19" t="s">
-        <v>65</v>
-      </c>
-      <c r="B19" t="s">
-        <v>66</v>
-      </c>
-    </row>
+    <row r="19" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="20" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="21" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="22" spans="1:2" ht="14.25" customHeight="1"/>
@@ -1753,7 +1740,6 @@
     <row r="996" ht="14.25" customHeight="1"/>
     <row r="997" ht="14.25" customHeight="1"/>
     <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added Document Understanding extraction flow
</commit_message>
<xml_diff>
--- a/RegEx Document Processing Demo/Data/Config.xlsx
+++ b/RegEx Document Processing Demo/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci\Documents\UiPath\REPO\RegEx Document Processing Demo\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC814826-A9B2-49E2-8728-1A02102AAB75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB594ED-A4F4-4FC9-9E03-DB69F15F7E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,13 +16,15 @@
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
     <sheet name="Constants" sheetId="2" r:id="rId2"/>
     <sheet name="Assets" sheetId="3" r:id="rId3"/>
+    <sheet name="InvoicePostProcessing" sheetId="4" r:id="rId4"/>
+    <sheet name="AutocorrectOcrMistakes" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="299">
   <si>
     <t>Name</t>
   </si>
@@ -220,13 +222,715 @@
   </si>
   <si>
     <t>RegEx_Footer_Order</t>
+  </si>
+  <si>
+    <t>ClassifierLearningFilePath</t>
+  </si>
+  <si>
+    <t>DocumentProcessing\IntelligentKeywordLearningFile.json</t>
+  </si>
+  <si>
+    <t>Path to the learning file of the classifier</t>
+  </si>
+  <si>
+    <t>UiPathOcrEndpoint</t>
+  </si>
+  <si>
+    <t>https://du.uipath.com/ocr</t>
+  </si>
+  <si>
+    <t>UiPath public endpoint for DocumentOCR</t>
+  </si>
+  <si>
+    <t>ReceiptsEndpoint</t>
+  </si>
+  <si>
+    <t>https://du.uipath.com/ie/receipts</t>
+  </si>
+  <si>
+    <t>UiPath public endpoint for receipts</t>
+  </si>
+  <si>
+    <t>InvoicesEndpoint</t>
+  </si>
+  <si>
+    <t>https://du.uipath.com/ie/invoices</t>
+  </si>
+  <si>
+    <t>UiPath public endpoint for invoices</t>
+  </si>
+  <si>
+    <t>ClassificationEndpoint</t>
+  </si>
+  <si>
+    <t>https://du.uipath.com/svc/intelligentkeywords</t>
+  </si>
+  <si>
+    <t>UiPath public endpoint for classification</t>
+  </si>
+  <si>
+    <t>FormExtractorEndpoint</t>
+  </si>
+  <si>
+    <t>https://du.uipath.com/svc/formextractor</t>
+  </si>
+  <si>
+    <t>UiPath public endpoint for Form Extractor</t>
+  </si>
+  <si>
+    <t>AlwaysValidateClassification</t>
+  </si>
+  <si>
+    <t>True</t>
+  </si>
+  <si>
+    <t>If set to True, classification will always go through manual validation. Has a corresponding asset that can be configured to overwrite this setting.</t>
+  </si>
+  <si>
+    <t>AlwaysValidateExtraction</t>
+  </si>
+  <si>
+    <t>If set to True, extracted data will always go through manual validation. Has a corresponding asset that can be configured to overwrite this setting.</t>
+  </si>
+  <si>
+    <t>SkipClassifierTraining</t>
+  </si>
+  <si>
+    <t>False</t>
+  </si>
+  <si>
+    <t>If set to True, classifier training will not be performed. Has a corresponding asset that can be configured to overwrite this setting.</t>
+  </si>
+  <si>
+    <t>SkipExtractorTraining</t>
+  </si>
+  <si>
+    <t>If set to True, extractor training will not be performed. Has a corresponding asset that can be configured to overwrite this setting.</t>
+  </si>
+  <si>
+    <t>ClassificationThreshold</t>
+  </si>
+  <si>
+    <t>Classification threshold for Classification Business Rule Validation must be a value between 0 and 1.</t>
+  </si>
+  <si>
+    <t>TargetFileKey</t>
+  </si>
+  <si>
+    <t>TargetFile</t>
+  </si>
+  <si>
+    <t>Key in the Transaction Item's dictionary that holds the path to the file to be processed</t>
+  </si>
+  <si>
+    <t>DU_DateFormats</t>
+  </si>
+  <si>
+    <t>yyyy-MM-dd;dd-MM-yyyy;MM-dd-yyyy;MM/dd/yyyy;dd/MM/yyyy;yyyy/MM/dd;dd.MM.yyyy;MM.dd.yyyy;yyyy.MM.dd</t>
+  </si>
+  <si>
+    <t>Different date formats.</t>
+  </si>
+  <si>
+    <t>ActionCatalog</t>
+  </si>
+  <si>
+    <t>Action Catalog Name. Has a corresponding asset that can be configured to overwrite this setting.</t>
+  </si>
+  <si>
+    <t>ActionFolderPath</t>
+  </si>
+  <si>
+    <t>Path to the Orchestrator Folder where the Action Catalog resides. Has a corresponding asset that can be configured to overwrite this setting.</t>
+  </si>
+  <si>
+    <t>StorageBucketName</t>
+  </si>
+  <si>
+    <t>Storage Bucket Name (required when Action Center is used). Has a corresponding asset that can be configured to overwrite this setting.</t>
+  </si>
+  <si>
+    <t>StorageBucketDirectoryPath</t>
+  </si>
+  <si>
+    <t>Path inside  the Storage Bucket where actions will store the files. Has a corresponding asset that can be configured to overwrite this setting.</t>
+  </si>
+  <si>
+    <t>DocumentUnderstandingQueueName</t>
+  </si>
+  <si>
+    <t>DU_InputQueue</t>
+  </si>
+  <si>
+    <t>The name of the Orchestrator Queue. Has a corresponding asset that can be configured to overwrite this setting.</t>
+  </si>
+  <si>
+    <t>DocumentUnderstandingQueuePath</t>
+  </si>
+  <si>
+    <t>Path to the Orchestrator Folder where the Queue resides. Has a corresponding asset that can be configured to overwrite this setting.</t>
+  </si>
+  <si>
+    <t>MaxExecutionAttempts</t>
+  </si>
+  <si>
+    <t>Maximum number of execution attempts for a process step. Minimum value is 1.</t>
+  </si>
+  <si>
+    <t>MaxExecutionAttemptsDigitize</t>
+  </si>
+  <si>
+    <t>Maximum number of execution attempts for the Digitize step. Minimum value is 1.  An OCR engine that uses a paid license might incur extra costs when re-executing. This should be taken into consideration when for the number of retries.</t>
+  </si>
+  <si>
+    <t>MaxExecutionAttemptsClassify</t>
+  </si>
+  <si>
+    <t>Maximum number of execution attempts for the Classify step. Minimum value is 1. A Classifier that uses a paid license might incur extra costs when re-executing. This should be taken into consideration when for the number of retries.</t>
+  </si>
+  <si>
+    <t>MaxExecutionAttemptsExtract</t>
+  </si>
+  <si>
+    <t>Maximum number of execution attempts for the Extract step. Minimum value is 1. An Extractor that uses a paid license might incur extra costs when re-executing. This should be taken into consideration for the number of retries.</t>
+  </si>
+  <si>
+    <t>MaxExecutionAttemptsHigh</t>
+  </si>
+  <si>
+    <t>Maximum number of execution attempts for a process step which by default is high.</t>
+  </si>
+  <si>
+    <t>MaxLockTimeout</t>
+  </si>
+  <si>
+    <t>Duration, in seconds, for how long will a job try to lock a training file before giving up and abandoning the training.</t>
+  </si>
+  <si>
+    <t>RetryInterval</t>
+  </si>
+  <si>
+    <t>Duration, in seconds, between re-execution attempts</t>
+  </si>
+  <si>
+    <t>RetryIntervalLow</t>
+  </si>
+  <si>
+    <t>ClassificationActionTitle</t>
+  </si>
+  <si>
+    <t>Classify -</t>
+  </si>
+  <si>
+    <t>ValidationActionTitle</t>
+  </si>
+  <si>
+    <t>Validate -</t>
+  </si>
+  <si>
+    <t>LogMessage_DocumentToProcess</t>
+  </si>
+  <si>
+    <t>Processing document:</t>
+  </si>
+  <si>
+    <t>LogMessage_InitStarted</t>
+  </si>
+  <si>
+    <t>Project initialization started</t>
+  </si>
+  <si>
+    <t>LogMessage_DigitizationStarted</t>
+  </si>
+  <si>
+    <t>Digitization started for:</t>
+  </si>
+  <si>
+    <t>LogMessage_DigitizationFinished</t>
+  </si>
+  <si>
+    <t>Digitization finished</t>
+  </si>
+  <si>
+    <t>LogMessage_AutoClassificationStarted</t>
+  </si>
+  <si>
+    <t>Automatic classification started</t>
+  </si>
+  <si>
+    <t>LogMessage_ClassificationFinished</t>
+  </si>
+  <si>
+    <t>Classification finished</t>
+  </si>
+  <si>
+    <t>LogMessage_AutoClassificationResults</t>
+  </si>
+  <si>
+    <t>Automatic classification results:</t>
+  </si>
+  <si>
+    <t>LogMessage_CreateClassificationAction</t>
+  </si>
+  <si>
+    <t>Creating classification validation action</t>
+  </si>
+  <si>
+    <t>LogMessage_WaitOnClassificationAction</t>
+  </si>
+  <si>
+    <t>Waiting on classification validation action #</t>
+  </si>
+  <si>
+    <t>LogMessage_ShowClassificationStation</t>
+  </si>
+  <si>
+    <t>Presenting Classification Station</t>
+  </si>
+  <si>
+    <t>LogMessage_ResumeAfterClassificationValidation</t>
+  </si>
+  <si>
+    <t>Resuming after classification validation{0}. Document(s) classified as: {1}</t>
+  </si>
+  <si>
+    <t>LogMessage_TrainClassifiersStart</t>
+  </si>
+  <si>
+    <t>Train classifiers started</t>
+  </si>
+  <si>
+    <t>LogMessage_ClassifierTrainingUnsuccessful</t>
+  </si>
+  <si>
+    <t>Classification retraining failed</t>
+  </si>
+  <si>
+    <t>LogMessage_ClassifierTrainingSuccessful</t>
+  </si>
+  <si>
+    <t>Classifiers trained successfully</t>
+  </si>
+  <si>
+    <t>LogMessage_DataExtractionStart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data extraction started for: </t>
+  </si>
+  <si>
+    <t>LogMessage_DataExtractionFinished</t>
+  </si>
+  <si>
+    <t>Data extraction finished</t>
+  </si>
+  <si>
+    <t>LogMessage_CreateValidationAction</t>
+  </si>
+  <si>
+    <t>Creating data validation action for:</t>
+  </si>
+  <si>
+    <t>LogMessage_WaitOnValidationAction</t>
+  </si>
+  <si>
+    <t>Waiting on data validation action #</t>
+  </si>
+  <si>
+    <t>LogMessage_ShowValidationStation</t>
+  </si>
+  <si>
+    <t>Presenting Validation Station for:</t>
+  </si>
+  <si>
+    <t>LogMessage_ResumeAfterDataValidation</t>
+  </si>
+  <si>
+    <t>Resuming after data validation{0}. Document: {1}</t>
+  </si>
+  <si>
+    <t>LogMessage_TrainExtractorsStart</t>
+  </si>
+  <si>
+    <t>Train extractors started</t>
+  </si>
+  <si>
+    <t>LogMessage_AutocorrectOcrMistakesStart</t>
+  </si>
+  <si>
+    <t>OCR Autocorrection started</t>
+  </si>
+  <si>
+    <t>LogMessage_AutocorrectOcrMistakesFinished</t>
+  </si>
+  <si>
+    <t>OCR Autocorrection finished</t>
+  </si>
+  <si>
+    <t>LogMessage_DataExportStart</t>
+  </si>
+  <si>
+    <t>Data export started for:</t>
+  </si>
+  <si>
+    <t>LogMessage_EndProcessStart</t>
+  </si>
+  <si>
+    <t>End process started</t>
+  </si>
+  <si>
+    <t>LogMessage_ExtractionBusinessRuleValidationStart</t>
+  </si>
+  <si>
+    <t>Extraction Business Rule Validation started for:</t>
+  </si>
+  <si>
+    <t>LogMessage_ClassificationBusinessRuleValidationStart</t>
+  </si>
+  <si>
+    <t>Classification Business Rule Validation started for:</t>
+  </si>
+  <si>
+    <t>LogMessage_GetWritePermission</t>
+  </si>
+  <si>
+    <t>Getting file write permission</t>
+  </si>
+  <si>
+    <t>LogMessage_GiveUpWritePermission</t>
+  </si>
+  <si>
+    <t>Giving up file write permission</t>
+  </si>
+  <si>
+    <t>LogMessage_LockFile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Locking keyword file: </t>
+  </si>
+  <si>
+    <t>LogMessage_UnLockFileStarted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unlocking keyword file: </t>
+  </si>
+  <si>
+    <t>LogMessage_UnLockFileFinished</t>
+  </si>
+  <si>
+    <t>Unlock complete!</t>
+  </si>
+  <si>
+    <t>LogMessage_GetTransactionItem</t>
+  </si>
+  <si>
+    <t>Get Transaction Item started</t>
+  </si>
+  <si>
+    <t>LogMessage_TransactionItemNotFound</t>
+  </si>
+  <si>
+    <t>No transaction item found in the queue</t>
+  </si>
+  <si>
+    <t>LogMessage_TargetFileMissingInTransactionItem</t>
+  </si>
+  <si>
+    <t>Transaction Item does not specify the file to be processed</t>
+  </si>
+  <si>
+    <t>LogMessage_SetTransactionStatusSuccess</t>
+  </si>
+  <si>
+    <t>Transaction Successful</t>
+  </si>
+  <si>
+    <t>LogMessage_SetTransactionStatusBRE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transaction failed due to Business Rule Exception: </t>
+  </si>
+  <si>
+    <t>LogMessage_SetTransactionStatusSystemException</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transaction failed due to System Exception: </t>
+  </si>
+  <si>
+    <t>LogMessage_SetTransactionProgress</t>
+  </si>
+  <si>
+    <t>Updating transaction progress to:</t>
+  </si>
+  <si>
+    <t>TransactionProgress_ClassificationValidation</t>
+  </si>
+  <si>
+    <t>Validating Classification</t>
+  </si>
+  <si>
+    <t>TransactionProgress_ExtractionValidation</t>
+  </si>
+  <si>
+    <t>Validating Extracted Data</t>
+  </si>
+  <si>
+    <t>WarnMessage_DocumentProcessingFailure</t>
+  </si>
+  <si>
+    <t>Failed to process page range {0} in file {1} due to {2} with message: {3} Full Exception: {4}</t>
+  </si>
+  <si>
+    <t>ErrorMessage_InputDocumentNotFound</t>
+  </si>
+  <si>
+    <t>Cannot find input document:</t>
+  </si>
+  <si>
+    <t>ErrorMessage_AssetFailedToLoad</t>
+  </si>
+  <si>
+    <t>Failed to load asset:</t>
+  </si>
+  <si>
+    <t>ErrorMessage_ProcessAborted</t>
+  </si>
+  <si>
+    <t>Process was aborted due to {0} with message: {1} Full Exception: {2}</t>
+  </si>
+  <si>
+    <t>ApiKey</t>
+  </si>
+  <si>
+    <t>DocumentUnderstandingApiKey</t>
+  </si>
+  <si>
+    <t>Retrieve your DocumentUnderstanding ApiKey and configure it in an Asset</t>
+  </si>
+  <si>
+    <t>If set to True, classification will always go through manual validation. Asset value overwrites the one from the "Settings" sheet</t>
+  </si>
+  <si>
+    <t>If set to True, extracted data will always go through manual validation. Asset value overwrites the one from the "Settings" sheet</t>
+  </si>
+  <si>
+    <t>If set to True, classifier training will not be performed. Asset value overwrites the one from the "Settings" sheet</t>
+  </si>
+  <si>
+    <t>If set to True, extractor training will not be performed. Asset value overwrites the one from the "Settings" sheet</t>
+  </si>
+  <si>
+    <t>DU_ActionCatalogName</t>
+  </si>
+  <si>
+    <t>Action Catalog Name. The asset value overrides the one from the "Settings" sheet</t>
+  </si>
+  <si>
+    <t>DU_ActionFolderPath</t>
+  </si>
+  <si>
+    <t>Path to the Orchestrator Folder where the Action Catalog resides. The asset value overrides the one from the "Settings" sheet</t>
+  </si>
+  <si>
+    <t>DU_StorageBucketName</t>
+  </si>
+  <si>
+    <t>Storage Bucket Name (required when Action Center is used). The asset value overrides the one from the "Settings" sheet</t>
+  </si>
+  <si>
+    <t>DU_StorageBucketDirectoryPath</t>
+  </si>
+  <si>
+    <t>Path inside  the Storage Bucket where actions will store the files. The asset value overrides the one from the "Settings" sheet</t>
+  </si>
+  <si>
+    <t>DU_QueueName</t>
+  </si>
+  <si>
+    <t>The name of the Orchestrator Queue. The asset value overrides the one from the "Settings" sheet</t>
+  </si>
+  <si>
+    <t>DU_QueuePath</t>
+  </si>
+  <si>
+    <t>Path to the Orchestrator Folder where the Queue resides. The asset value overrides the one from the "Settings" sheet</t>
+  </si>
+  <si>
+    <t>DU_ClassificationThreshold</t>
+  </si>
+  <si>
+    <t>AutocorrectStorageBucketDirectoryPath</t>
+  </si>
+  <si>
+    <t>DU_AutocorrectStorageBucketDirectoryPath</t>
+  </si>
+  <si>
+    <t>Path inside the Storage Bucket where the autocorrect file is stored. The asset value overrides the one from the "AutocorrectOcrMistakes" sheet</t>
+  </si>
+  <si>
+    <t>MinimumNumberOfRepetitions</t>
+  </si>
+  <si>
+    <t>DU_MinimumNumberOfRepetitions</t>
+  </si>
+  <si>
+    <t>The minimum number of times the value needs to be corrected in Action Center before the flow will start to autocorrect. The asset value overrides the one from the "AutocorrectOcrMistakes" sheet</t>
+  </si>
+  <si>
+    <t>AutocorrectionEnabled</t>
+  </si>
+  <si>
+    <t>DU_AutocorrectionEnabled</t>
+  </si>
+  <si>
+    <t>A flag that determines if autocorrection should be called or not. The asset value overrides the one from the "AutocorrectOcrMistakes" sheet</t>
+  </si>
+  <si>
+    <t>AutocorrectionFieldIdList</t>
+  </si>
+  <si>
+    <t>DU_AutocorrectionFieldIdList</t>
+  </si>
+  <si>
+    <t>A comma separated list of the taxonomy ids of the fields we want to enable autocorrection for. Has a corresponding asset that can be configured to overwrite this setting.</t>
+  </si>
+  <si>
+    <t>LogMessage_InvoicePostProcessing</t>
+  </si>
+  <si>
+    <t>Starting Invoice Post Processing</t>
+  </si>
+  <si>
+    <t>LogMessage_InvoicePostProcessing_DateFailure</t>
+  </si>
+  <si>
+    <t>Parsing the Date has failed!</t>
+  </si>
+  <si>
+    <t>LogMessage_InvoicePostProcessing_MandatoryFieldsFailure</t>
+  </si>
+  <si>
+    <t>One or more of the mandatory were missing!</t>
+  </si>
+  <si>
+    <t>LogMessage_InvoicePostProcessing_LineAmountFailureMath</t>
+  </si>
+  <si>
+    <t>Quantity * Unit-price is not equal to Line Amount!</t>
+  </si>
+  <si>
+    <t>LogMessage_InvoicePostProcessing_LineAmountFailureEmpty</t>
+  </si>
+  <si>
+    <t>Quantity or Unit-price is Empty!</t>
+  </si>
+  <si>
+    <t>LogMessage_InvoicePostProcessing_AlreadySetFalse</t>
+  </si>
+  <si>
+    <t>AutoExtraction is already set to false in a previous step. Skipping rest of checks.</t>
+  </si>
+  <si>
+    <t>LogMessage_InvoicePostProcessing_SubtotalFailure</t>
+  </si>
+  <si>
+    <t>Subtotal Failure with subtotal: {0} and net-amount {1}</t>
+  </si>
+  <si>
+    <t>LogMessage_InvoicePostProcessing_TotalFailure</t>
+  </si>
+  <si>
+    <t>Total Computation Failed!</t>
+  </si>
+  <si>
+    <t>LogMessage_InvoicePostProcessing_SubtotalPass</t>
+  </si>
+  <si>
+    <t>Subtotal Pass with subtotal: {0} and net-amount {1}</t>
+  </si>
+  <si>
+    <t>LogMessage_InvoicePostProcessing_ConfidenceFieldsFailure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">These are the fields that failed: </t>
+  </si>
+  <si>
+    <t>SubTotalAdditions</t>
+  </si>
+  <si>
+    <t>Tax Amount,Shipping Charges,Discount</t>
+  </si>
+  <si>
+    <t>Each field present in the list here, will be added to the subtotal to compute the total</t>
+  </si>
+  <si>
+    <t>MandatoryFields</t>
+  </si>
+  <si>
+    <t>Date,Invoice Number,PO Number,Total</t>
+  </si>
+  <si>
+    <t>These fields are mandatory. If they have not been extracted at all, the document will be sent for validation</t>
+  </si>
+  <si>
+    <t>MandatoryColumnFields</t>
+  </si>
+  <si>
+    <t>Quantity,Unit Price,Line Amount</t>
+  </si>
+  <si>
+    <t>These column fields are mandatory. If they have not been extracted at all, the document will be sent for validation</t>
+  </si>
+  <si>
+    <t>ConfidenceFields</t>
+  </si>
+  <si>
+    <t>Date,Shipping Address,Invoice Number,PO Number</t>
+  </si>
+  <si>
+    <t>List of fields which will be checked versus a specific confidence threshold. All new entries must have the "-Confidence" suffix</t>
+  </si>
+  <si>
+    <t>OtherConfidenceFields</t>
+  </si>
+  <si>
+    <t>Tax Amount,Net Amount,Discount,Shipping Charges,Billing Name,Total, Name, Vendor Address, Billing Address, Billing VAT Number, Payment Address, Vendor VAT Number, DueDate,Payment Terms</t>
+  </si>
+  <si>
+    <t>List of fields which will be checked versus a single confidence #:  Other-Confidence</t>
+  </si>
+  <si>
+    <t>Date-Confidence</t>
+  </si>
+  <si>
+    <t>Shipping Address-Confidence</t>
+  </si>
+  <si>
+    <t>Invoice Number-Confidence</t>
+  </si>
+  <si>
+    <t>PO Number-Confidence</t>
+  </si>
+  <si>
+    <t>other-Confidence</t>
+  </si>
+  <si>
+    <t>AutocorrectionLearningFile.json</t>
+  </si>
+  <si>
+    <t>Path inside the Storage Bucket where the autocorrect file is stored. Has a corresponding asset that can be configured to overwrite this setting.</t>
+  </si>
+  <si>
+    <t>The minimum number of times the value needs to be corrected in Action Center before the flow will start to autocorrect. Has a corresponding asset that can be configured to overwrite this setting.</t>
+  </si>
+  <si>
+    <t>A flag that determines if autocorrection should be called or not. Has a corresponding asset that can be configured to overwrite this setting.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -256,6 +960,32 @@
       <family val="2"/>
       <charset val="238"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -274,10 +1004,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -288,8 +1019,14 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperłącze" xfId="1" builtinId="8"/>
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -751,8 +1488,8 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="18" spans="1:2" ht="14.25" customHeight="1">
+    <row r="17" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="18" spans="1:3" ht="14.25" customHeight="1">
       <c r="A18" t="s">
         <v>56</v>
       </c>
@@ -760,36 +1497,223 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="20" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="21" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="22" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="23" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="24" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="25" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="26" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="27" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="28" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="29" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="30" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="31" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="32" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="33" ht="14.25" customHeight="1"/>
-    <row r="34" ht="14.25" customHeight="1"/>
-    <row r="35" ht="14.25" customHeight="1"/>
-    <row r="36" ht="14.25" customHeight="1"/>
-    <row r="37" ht="14.25" customHeight="1"/>
-    <row r="38" ht="14.25" customHeight="1"/>
-    <row r="39" ht="14.25" customHeight="1"/>
-    <row r="40" ht="14.25" customHeight="1"/>
-    <row r="41" ht="14.25" customHeight="1"/>
-    <row r="42" ht="14.25" customHeight="1"/>
-    <row r="43" ht="14.25" customHeight="1"/>
-    <row r="44" ht="14.25" customHeight="1"/>
-    <row r="45" ht="14.25" customHeight="1"/>
-    <row r="46" ht="14.25" customHeight="1"/>
-    <row r="47" ht="14.25" customHeight="1"/>
-    <row r="48" ht="14.25" customHeight="1"/>
+    <row r="19" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A20" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="22" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A22" t="s">
+        <v>68</v>
+      </c>
+      <c r="B22" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A23" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" t="s">
+        <v>72</v>
+      </c>
+      <c r="C23" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A24" t="s">
+        <v>74</v>
+      </c>
+      <c r="B24" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A25" t="s">
+        <v>77</v>
+      </c>
+      <c r="B25" t="s">
+        <v>78</v>
+      </c>
+      <c r="C25" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A26" t="s">
+        <v>80</v>
+      </c>
+      <c r="B26" t="s">
+        <v>81</v>
+      </c>
+      <c r="C26" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A32" s="2"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="2"/>
+    </row>
+    <row r="33" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A33" t="s">
+        <v>93</v>
+      </c>
+      <c r="B33">
+        <v>0.5</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="14.25" customHeight="1">
+      <c r="C34" s="2"/>
+    </row>
+    <row r="35" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A35" t="s">
+        <v>95</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C35" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B36" s="2"/>
+    </row>
+    <row r="37" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A37" t="s">
+        <v>98</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C37" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B38" s="2"/>
+    </row>
+    <row r="39" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A39" t="s">
+        <v>101</v>
+      </c>
+      <c r="B39" s="2"/>
+      <c r="C39" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A40" t="s">
+        <v>103</v>
+      </c>
+      <c r="C40" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A41" t="s">
+        <v>105</v>
+      </c>
+      <c r="B41" s="2"/>
+      <c r="C41" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A42" t="s">
+        <v>107</v>
+      </c>
+      <c r="C42" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A43" t="s">
+        <v>109</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C43" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A44" t="s">
+        <v>112</v>
+      </c>
+      <c r="C44" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="46" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="47" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="48" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="49" ht="14.25" customHeight="1"/>
     <row r="50" ht="14.25" customHeight="1"/>
     <row r="51" ht="14.25" customHeight="1"/>
@@ -1929,84 +2853,493 @@
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="19" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="22" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="24" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="25" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="26" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="19" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A19" t="s">
+        <v>114</v>
+      </c>
+      <c r="B19">
+        <v>3</v>
+      </c>
+      <c r="C19" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A20" t="s">
+        <v>116</v>
+      </c>
+      <c r="B20">
+        <v>3</v>
+      </c>
+      <c r="C20" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A21" t="s">
+        <v>118</v>
+      </c>
+      <c r="B21">
+        <v>3</v>
+      </c>
+      <c r="C21" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B22">
+        <v>3</v>
+      </c>
+      <c r="C22" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A23" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23">
+        <v>99999</v>
+      </c>
+      <c r="C23" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A24" t="s">
+        <v>124</v>
+      </c>
+      <c r="B24">
+        <v>30</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A25" t="s">
+        <v>126</v>
+      </c>
+      <c r="B25">
+        <v>30</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A26" t="s">
+        <v>128</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="28" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="29" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A28" t="s">
+        <v>129</v>
+      </c>
+      <c r="B28" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A29" t="s">
+        <v>131</v>
+      </c>
+      <c r="B29" t="s">
+        <v>132</v>
+      </c>
+    </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="31" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="32" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="33" ht="14.25" customHeight="1"/>
-    <row r="34" ht="14.25" customHeight="1"/>
-    <row r="35" ht="14.25" customHeight="1"/>
-    <row r="36" ht="14.25" customHeight="1"/>
-    <row r="37" ht="14.25" customHeight="1"/>
-    <row r="38" ht="14.25" customHeight="1"/>
-    <row r="39" ht="14.25" customHeight="1"/>
-    <row r="40" ht="14.25" customHeight="1"/>
-    <row r="41" ht="14.25" customHeight="1"/>
-    <row r="42" ht="14.25" customHeight="1"/>
-    <row r="43" ht="14.25" customHeight="1"/>
-    <row r="44" ht="14.25" customHeight="1"/>
-    <row r="45" ht="14.25" customHeight="1"/>
-    <row r="46" ht="14.25" customHeight="1"/>
-    <row r="47" ht="14.25" customHeight="1"/>
-    <row r="48" ht="14.25" customHeight="1"/>
-    <row r="49" ht="14.25" customHeight="1"/>
-    <row r="50" ht="14.25" customHeight="1"/>
-    <row r="51" ht="14.25" customHeight="1"/>
-    <row r="52" ht="14.25" customHeight="1"/>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
-    <row r="57" ht="14.25" customHeight="1"/>
-    <row r="58" ht="14.25" customHeight="1"/>
-    <row r="59" ht="14.25" customHeight="1"/>
-    <row r="60" ht="14.25" customHeight="1"/>
-    <row r="61" ht="14.25" customHeight="1"/>
-    <row r="62" ht="14.25" customHeight="1"/>
-    <row r="63" ht="14.25" customHeight="1"/>
-    <row r="64" ht="14.25" customHeight="1"/>
-    <row r="65" ht="14.25" customHeight="1"/>
-    <row r="66" ht="14.25" customHeight="1"/>
-    <row r="67" ht="14.25" customHeight="1"/>
-    <row r="68" ht="14.25" customHeight="1"/>
-    <row r="69" ht="14.25" customHeight="1"/>
-    <row r="70" ht="14.25" customHeight="1"/>
-    <row r="71" ht="14.25" customHeight="1"/>
-    <row r="72" ht="14.25" customHeight="1"/>
-    <row r="73" ht="14.25" customHeight="1"/>
-    <row r="74" ht="14.25" customHeight="1"/>
-    <row r="75" ht="14.25" customHeight="1"/>
-    <row r="76" ht="14.25" customHeight="1"/>
-    <row r="77" ht="14.25" customHeight="1"/>
-    <row r="78" ht="14.25" customHeight="1"/>
-    <row r="79" ht="14.25" customHeight="1"/>
-    <row r="80" ht="14.25" customHeight="1"/>
-    <row r="81" ht="14.25" customHeight="1"/>
-    <row r="82" ht="14.25" customHeight="1"/>
-    <row r="83" ht="14.25" customHeight="1"/>
-    <row r="84" ht="14.25" customHeight="1"/>
-    <row r="85" ht="14.25" customHeight="1"/>
-    <row r="86" ht="14.25" customHeight="1"/>
-    <row r="87" ht="14.25" customHeight="1"/>
-    <row r="88" ht="14.25" customHeight="1"/>
-    <row r="89" ht="14.25" customHeight="1"/>
-    <row r="90" ht="14.25" customHeight="1"/>
-    <row r="91" ht="14.25" customHeight="1"/>
-    <row r="92" ht="14.25" customHeight="1"/>
-    <row r="93" ht="14.25" customHeight="1"/>
-    <row r="94" ht="14.25" customHeight="1"/>
-    <row r="95" ht="14.25" customHeight="1"/>
-    <row r="96" ht="14.25" customHeight="1"/>
+    <row r="31" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A31" t="s">
+        <v>133</v>
+      </c>
+      <c r="B31" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A32" t="s">
+        <v>135</v>
+      </c>
+      <c r="B32" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A33" t="s">
+        <v>137</v>
+      </c>
+      <c r="B33" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A34" t="s">
+        <v>139</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A35" t="s">
+        <v>141</v>
+      </c>
+      <c r="B35" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A36" t="s">
+        <v>143</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A37" t="s">
+        <v>145</v>
+      </c>
+      <c r="B37" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A38" t="s">
+        <v>147</v>
+      </c>
+      <c r="B38" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A39" t="s">
+        <v>149</v>
+      </c>
+      <c r="B39" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A40" t="s">
+        <v>151</v>
+      </c>
+      <c r="B40" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A41" t="s">
+        <v>153</v>
+      </c>
+      <c r="B41" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A42" t="s">
+        <v>155</v>
+      </c>
+      <c r="B42" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A43" t="s">
+        <v>157</v>
+      </c>
+      <c r="B43" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A44" t="s">
+        <v>159</v>
+      </c>
+      <c r="B44" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A45" t="s">
+        <v>161</v>
+      </c>
+      <c r="B45" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A47" t="s">
+        <v>165</v>
+      </c>
+      <c r="B47" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A48" t="s">
+        <v>167</v>
+      </c>
+      <c r="B48" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A49" t="s">
+        <v>169</v>
+      </c>
+      <c r="B49" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A50" t="s">
+        <v>171</v>
+      </c>
+      <c r="B50" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A51" t="s">
+        <v>173</v>
+      </c>
+      <c r="B51" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A52" t="s">
+        <v>175</v>
+      </c>
+      <c r="B52" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A53" t="s">
+        <v>177</v>
+      </c>
+      <c r="B53" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A54" t="s">
+        <v>179</v>
+      </c>
+      <c r="B54" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A55" t="s">
+        <v>181</v>
+      </c>
+      <c r="B55" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="59" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A59" t="s">
+        <v>187</v>
+      </c>
+      <c r="B59" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A60" t="s">
+        <v>189</v>
+      </c>
+      <c r="B60" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="62" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A62" t="s">
+        <v>191</v>
+      </c>
+      <c r="B62" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A63" t="s">
+        <v>193</v>
+      </c>
+      <c r="B63" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A64" t="s">
+        <v>195</v>
+      </c>
+      <c r="B64" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="66" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A66" t="s">
+        <v>197</v>
+      </c>
+      <c r="B66" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A67" t="s">
+        <v>199</v>
+      </c>
+      <c r="B67" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A68" t="s">
+        <v>201</v>
+      </c>
+      <c r="B68" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A69" t="s">
+        <v>203</v>
+      </c>
+      <c r="B69" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A70" t="s">
+        <v>205</v>
+      </c>
+      <c r="B70" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A71" t="s">
+        <v>207</v>
+      </c>
+      <c r="B71" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A72" t="s">
+        <v>209</v>
+      </c>
+      <c r="B72" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="74" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A74" t="s">
+        <v>211</v>
+      </c>
+      <c r="B74" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A75" t="s">
+        <v>213</v>
+      </c>
+      <c r="B75" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="77" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A77" t="s">
+        <v>215</v>
+      </c>
+      <c r="B77" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="79" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A79" t="s">
+        <v>217</v>
+      </c>
+      <c r="B79" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A80" t="s">
+        <v>219</v>
+      </c>
+      <c r="B80" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A81" t="s">
+        <v>221</v>
+      </c>
+      <c r="B81" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="83" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="84" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="85" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="86" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="87" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="88" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="89" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="90" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="91" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="92" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="93" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="94" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="95" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="96" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="97" ht="14.25" customHeight="1"/>
     <row r="98" ht="14.25" customHeight="1"/>
     <row r="99" ht="14.25" customHeight="1"/>
@@ -2952,37 +4285,211 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="3" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="2" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B2" t="s">
+        <v>224</v>
+      </c>
+      <c r="D2" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="D8" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="D9" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" t="s">
+        <v>234</v>
+      </c>
+      <c r="D10" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" t="s">
+        <v>107</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D11" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A12" t="s">
+        <v>109</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D12" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B13" t="s">
+        <v>240</v>
+      </c>
+      <c r="D13" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" ht="14.25" customHeight="1"/>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A16" t="s">
+        <v>243</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D16" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A17" t="s">
+        <v>246</v>
+      </c>
+      <c r="B17" t="s">
+        <v>247</v>
+      </c>
+      <c r="D17" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A18" t="s">
+        <v>249</v>
+      </c>
+      <c r="B18" t="s">
+        <v>250</v>
+      </c>
+      <c r="D18" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A19" t="s">
+        <v>252</v>
+      </c>
+      <c r="B19" t="s">
+        <v>253</v>
+      </c>
+      <c r="D19" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="21" spans="1:4" ht="14.25" customHeight="1">
+      <c r="A21" t="s">
+        <v>98</v>
+      </c>
+      <c r="B21" t="s">
+        <v>98</v>
+      </c>
+      <c r="D21" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="23" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="24" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="25" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="26" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="27" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="29" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="30" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="31" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="32" spans="1:4" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>
@@ -3955,4 +5462,1357 @@
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92A4CE3F-370D-498E-8CEC-17EC0E626FC8}">
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="57.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="72.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="115" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>255</v>
+      </c>
+      <c r="B3" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>257</v>
+      </c>
+      <c r="B4" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>259</v>
+      </c>
+      <c r="B5" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>261</v>
+      </c>
+      <c r="B6" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>263</v>
+      </c>
+      <c r="B7" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>265</v>
+      </c>
+      <c r="B8" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>267</v>
+      </c>
+      <c r="B9" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>269</v>
+      </c>
+      <c r="B10" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>271</v>
+      </c>
+      <c r="B11" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>273</v>
+      </c>
+      <c r="B13" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>275</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C15" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>278</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="C16" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>281</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="C17" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>284</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="C18" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>287</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="C19" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B21">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B22">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B23">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="B24">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>294</v>
+      </c>
+      <c r="B25">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5740500-B5EB-4696-A4C0-ED7892074369}">
+  <dimension ref="A1:Z1005"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="43.85546875" customWidth="1"/>
+    <col min="2" max="2" width="70.140625" customWidth="1"/>
+    <col min="3" max="3" width="166" bestFit="1" customWidth="1"/>
+    <col min="4" max="26" width="8.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
+      <c r="P1" s="8"/>
+      <c r="Q1" s="8"/>
+      <c r="R1" s="8"/>
+      <c r="S1" s="8"/>
+      <c r="T1" s="8"/>
+      <c r="U1" s="8"/>
+      <c r="V1" s="8"/>
+      <c r="W1" s="8"/>
+      <c r="X1" s="8"/>
+      <c r="Y1" s="8"/>
+      <c r="Z1" s="8"/>
+    </row>
+    <row r="2" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
+      <c r="P2" s="8"/>
+      <c r="Q2" s="8"/>
+      <c r="R2" s="8"/>
+      <c r="S2" s="8"/>
+      <c r="T2" s="8"/>
+      <c r="U2" s="8"/>
+      <c r="V2" s="8"/>
+      <c r="W2" s="8"/>
+      <c r="X2" s="8"/>
+      <c r="Y2" s="8"/>
+      <c r="Z2" s="8"/>
+    </row>
+    <row r="3" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A3" t="s">
+        <v>243</v>
+      </c>
+      <c r="B3" t="s">
+        <v>295</v>
+      </c>
+      <c r="C3" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="5" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A5" t="s">
+        <v>246</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" t="s">
+        <v>249</v>
+      </c>
+      <c r="B6" t="b">
+        <v>0</v>
+      </c>
+      <c r="C6" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" t="s">
+        <v>252</v>
+      </c>
+      <c r="C7" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A16" s="2"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A17" s="2"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A18" s="2"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A19" s="2"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A20" s="2"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1">
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3" ht="14.25" customHeight="1">
+      <c r="C22" s="2"/>
+    </row>
+    <row r="23" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B23" s="2"/>
+    </row>
+    <row r="24" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B24" s="2"/>
+    </row>
+    <row r="25" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B25" s="2"/>
+    </row>
+    <row r="26" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B27" s="2"/>
+    </row>
+    <row r="28" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="29" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B29" s="2"/>
+    </row>
+    <row r="30" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="32" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="33" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="34" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="35" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="36" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="37" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="38" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="39" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="40" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="41" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="42" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="43" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="44" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="45" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="46" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="47" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="48" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="49" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="50" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="51" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="52" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="53" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="54" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="55" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="56" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="57" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="58" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="59" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="60" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="61" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="62" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="63" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="64" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="65" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="66" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="67" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="68" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="69" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="70" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="71" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="72" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="73" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="74" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="75" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="76" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="77" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="78" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="79" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="80" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="81" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="82" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="83" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="84" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="85" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="86" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="87" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="88" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="89" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="90" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="91" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="92" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="93" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="94" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="95" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="96" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="97" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="98" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="99" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="100" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="101" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="102" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="103" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="104" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="105" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="106" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="107" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="108" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="109" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="110" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="111" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="112" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="113" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="114" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="115" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="116" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="117" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="118" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="119" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="120" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="121" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="122" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="123" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="124" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="125" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="126" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="127" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="128" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="129" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="130" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="131" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="132" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="133" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="134" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="135" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="136" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="137" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="138" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="139" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="140" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="141" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="142" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="143" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="144" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="145" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="146" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="147" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="148" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="149" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="150" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="151" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="152" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="153" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="154" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="155" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="156" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="157" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="158" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="159" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="160" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="161" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="162" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="163" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="164" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="165" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="166" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="167" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="168" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="169" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="170" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="171" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="172" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="173" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="174" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="175" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="176" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="177" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="178" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="179" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="180" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="181" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="182" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="183" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="184" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="185" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="186" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="187" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="188" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="189" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="190" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="191" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="192" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="193" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="194" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="195" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="196" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="197" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="198" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="199" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="200" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="201" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="202" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="203" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="204" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="205" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="206" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="207" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="208" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="209" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="210" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="211" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="212" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="213" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="214" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="215" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="216" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="217" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="218" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="219" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="220" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="221" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="222" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="223" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="224" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="225" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="226" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="227" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="228" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="229" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="230" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="231" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="232" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="233" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="234" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="235" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="236" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="237" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="238" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="239" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="240" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="241" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="242" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="243" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="244" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="245" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="246" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="247" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="248" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="249" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="250" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="251" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="252" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="253" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="254" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="255" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="256" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="257" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="258" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="259" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="260" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="261" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="262" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="263" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="264" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="265" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="266" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="267" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="268" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="269" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="270" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="271" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="272" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="273" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="274" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="275" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="276" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="277" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="278" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="279" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="280" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="281" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="282" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="283" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="284" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="285" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="286" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="287" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="288" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="289" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="290" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="291" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="292" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="293" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="294" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="295" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="296" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="297" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="298" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="299" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="300" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="301" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="302" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="303" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="304" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="305" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="306" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="307" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="308" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="309" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="310" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="311" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="312" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="313" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="314" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="315" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="316" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="317" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="318" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="319" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="320" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="321" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="322" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="323" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="324" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="325" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="326" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="327" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="328" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="329" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="330" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="331" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="332" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="333" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="334" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="335" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="336" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="337" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="338" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="339" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="340" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="341" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="342" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="343" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="344" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="345" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="346" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="347" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="348" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="349" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="350" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="351" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="352" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="353" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="354" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="355" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="356" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="357" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="358" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="359" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="360" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="361" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="362" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="363" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="364" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="365" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="366" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="367" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="368" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="369" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="370" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="371" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="372" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="373" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="374" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="375" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="376" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="377" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="378" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="379" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="380" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="381" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="382" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="383" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="384" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="385" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="386" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="387" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="388" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="389" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="390" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="391" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="392" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="393" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="394" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="395" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="396" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="397" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="398" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="399" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="400" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="401" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="402" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="403" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="404" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="405" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="406" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="407" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="408" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="409" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="410" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="411" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="412" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="413" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="414" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="415" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="416" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="417" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="418" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="419" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="420" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="421" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="422" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="423" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="424" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="425" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="426" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="427" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="428" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="429" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="430" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="431" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="432" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="433" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="434" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="435" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="436" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="437" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="438" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="439" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="440" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="441" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="442" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="443" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="444" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="445" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="446" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="447" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="448" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="449" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="450" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="451" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="452" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="453" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="454" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="455" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="456" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="457" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="458" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="459" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="460" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="461" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="462" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="463" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="464" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="465" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="466" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="467" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="468" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="469" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="470" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="471" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="472" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="473" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="474" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="475" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="476" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="477" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="478" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="479" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="480" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="481" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="482" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="483" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="484" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="485" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="486" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="487" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="488" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="489" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="490" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="491" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="492" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="493" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="494" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="495" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="496" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="497" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="498" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="499" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="500" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="501" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="502" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="503" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="504" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="505" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="506" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="507" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="508" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="509" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="510" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="511" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="512" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="513" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="514" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="515" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="516" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="517" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="518" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="519" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="520" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="521" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="522" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="523" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="524" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="525" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="526" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="527" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="528" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="529" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="530" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="531" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="532" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="533" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="534" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="535" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="536" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="537" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="538" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="539" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="540" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="541" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="542" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="543" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="544" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="545" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="546" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="547" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="548" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="549" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="550" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="551" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="552" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="553" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="554" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="555" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="556" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="557" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="558" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="559" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="560" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="561" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="562" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="563" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="564" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="565" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="566" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="567" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="568" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="569" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="570" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="571" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="572" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="573" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="574" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="575" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="576" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="577" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="578" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="579" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="580" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="581" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="582" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="583" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="584" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="585" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="586" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="587" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="588" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="589" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="590" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="591" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="592" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="593" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="594" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="595" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="596" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="597" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="598" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="599" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="600" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="601" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="602" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="603" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="604" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="605" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="606" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="607" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="608" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="609" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="610" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="611" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="612" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="613" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="614" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="615" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="616" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="617" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="618" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="619" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="620" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="621" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="622" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="623" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="624" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="625" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="626" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="627" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="628" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="629" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="630" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="631" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="632" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="633" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="634" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="635" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="636" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="637" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="638" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="639" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="640" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="641" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="642" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="643" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="644" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="645" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="646" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="647" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="648" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="649" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="650" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="651" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="652" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="653" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="654" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="655" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="656" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="657" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="658" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="659" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="660" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="661" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="662" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="663" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="664" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="665" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="666" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="667" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="668" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="669" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="670" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="671" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="672" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="673" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="674" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="675" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="676" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="677" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="678" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="679" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="680" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="681" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="682" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="683" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="684" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="685" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="686" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="687" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="688" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="689" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="690" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="691" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="692" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="693" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="694" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="695" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="696" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="697" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="698" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="699" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="700" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="701" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="702" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="703" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="704" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="705" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="706" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="707" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="708" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="709" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="710" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="711" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="712" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="713" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="714" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="715" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="716" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="717" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="718" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="719" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="720" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="721" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="722" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="723" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="724" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="725" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="726" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="727" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="728" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="729" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="730" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="731" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="732" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="733" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="734" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="735" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="736" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="737" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="738" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="739" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="740" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="741" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="742" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="743" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="744" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="745" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="746" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="747" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="748" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="749" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="750" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="751" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="752" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="753" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="754" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="755" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="756" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="757" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="758" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="759" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="760" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="761" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="762" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="763" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="764" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="765" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="766" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="767" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="768" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="769" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="770" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="771" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="772" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="773" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="774" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="775" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="776" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="777" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="778" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="779" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="780" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="781" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="782" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="783" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="784" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="785" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="786" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="787" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="788" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="789" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="790" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="791" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="792" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="793" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="794" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="795" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="796" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="797" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="798" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="799" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="800" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="801" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="802" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="803" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="804" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="805" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="806" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="807" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="808" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="809" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="810" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="811" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="812" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="813" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="814" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="815" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="816" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="817" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="818" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="819" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="820" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="821" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="822" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="823" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="824" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="825" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="826" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="827" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="828" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="829" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="830" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="831" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="832" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="833" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="834" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="835" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="836" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="837" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="838" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="839" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="840" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="841" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="842" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="843" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="844" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="845" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="846" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="847" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="848" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="849" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="850" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="851" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="852" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="853" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="854" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="855" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="856" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="857" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="858" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="859" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="860" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="861" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="862" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="863" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="864" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="865" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="866" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="867" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="868" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="869" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="870" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="871" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="872" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="873" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="874" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="875" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="876" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="877" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="878" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="879" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="880" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="881" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="882" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="883" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="884" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="885" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="886" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="887" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="888" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="889" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="890" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="891" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="892" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="893" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="894" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="895" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="896" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="897" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="898" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="899" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="900" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="901" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="902" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="903" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="904" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="905" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="906" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="907" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="908" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="909" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="910" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="911" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="912" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="913" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="914" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="915" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="916" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="917" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="918" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="919" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="920" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="921" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="922" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="923" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="924" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="925" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="926" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="927" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="928" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="929" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="930" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="931" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="932" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="933" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="934" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="935" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="936" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="937" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="938" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="939" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="940" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="941" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="942" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="943" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="944" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="945" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="946" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="947" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="948" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="949" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="950" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="951" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="952" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="953" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="954" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="955" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="956" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="957" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="958" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="959" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="960" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="961" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="962" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="963" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="964" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="965" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="966" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="967" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="968" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="969" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="970" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="971" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="972" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="973" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="974" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="975" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="976" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="977" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="978" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="979" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="980" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="981" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="982" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="983" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="984" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="985" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="986" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="987" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="988" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="989" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="990" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="991" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="992" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="993" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="994" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="995" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="996" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="997" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="998" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="999" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="1000" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="1001" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="1002" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="1003" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="1004" customFormat="1" ht="14.25" customHeight="1"/>
+    <row r="1005" customFormat="1" ht="14.25" customHeight="1"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Google Cloud integration
</commit_message>
<xml_diff>
--- a/RegEx Document Processing Demo/Data/Config.xlsx
+++ b/RegEx Document Processing Demo/Data/Config.xlsx
@@ -8,23 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci\Documents\UiPath\REPO\RegEx Document Processing Demo\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB594ED-A4F4-4FC9-9E03-DB69F15F7E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51AFD3D-FE7D-43D1-9E96-C1875C35E69A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
     <sheet name="Constants" sheetId="2" r:id="rId2"/>
-    <sheet name="Assets" sheetId="3" r:id="rId3"/>
-    <sheet name="InvoicePostProcessing" sheetId="4" r:id="rId4"/>
-    <sheet name="AutocorrectOcrMistakes" sheetId="5" r:id="rId5"/>
+    <sheet name="Assets" sheetId="6" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="227">
   <si>
     <t>Name</t>
   </si>
@@ -698,239 +696,23 @@
     <t>Process was aborted due to {0} with message: {1} Full Exception: {2}</t>
   </si>
   <si>
-    <t>ApiKey</t>
-  </si>
-  <si>
-    <t>DocumentUnderstandingApiKey</t>
-  </si>
-  <si>
-    <t>Retrieve your DocumentUnderstanding ApiKey and configure it in an Asset</t>
-  </si>
-  <si>
-    <t>If set to True, classification will always go through manual validation. Asset value overwrites the one from the "Settings" sheet</t>
-  </si>
-  <si>
-    <t>If set to True, extracted data will always go through manual validation. Asset value overwrites the one from the "Settings" sheet</t>
-  </si>
-  <si>
-    <t>If set to True, classifier training will not be performed. Asset value overwrites the one from the "Settings" sheet</t>
-  </si>
-  <si>
-    <t>If set to True, extractor training will not be performed. Asset value overwrites the one from the "Settings" sheet</t>
-  </si>
-  <si>
-    <t>DU_ActionCatalogName</t>
-  </si>
-  <si>
-    <t>Action Catalog Name. The asset value overrides the one from the "Settings" sheet</t>
-  </si>
-  <si>
-    <t>DU_ActionFolderPath</t>
-  </si>
-  <si>
-    <t>Path to the Orchestrator Folder where the Action Catalog resides. The asset value overrides the one from the "Settings" sheet</t>
-  </si>
-  <si>
-    <t>DU_StorageBucketName</t>
-  </si>
-  <si>
-    <t>Storage Bucket Name (required when Action Center is used). The asset value overrides the one from the "Settings" sheet</t>
-  </si>
-  <si>
-    <t>DU_StorageBucketDirectoryPath</t>
-  </si>
-  <si>
-    <t>Path inside  the Storage Bucket where actions will store the files. The asset value overrides the one from the "Settings" sheet</t>
-  </si>
-  <si>
-    <t>DU_QueueName</t>
-  </si>
-  <si>
-    <t>The name of the Orchestrator Queue. The asset value overrides the one from the "Settings" sheet</t>
-  </si>
-  <si>
-    <t>DU_QueuePath</t>
-  </si>
-  <si>
-    <t>Path to the Orchestrator Folder where the Queue resides. The asset value overrides the one from the "Settings" sheet</t>
-  </si>
-  <si>
-    <t>DU_ClassificationThreshold</t>
-  </si>
-  <si>
-    <t>AutocorrectStorageBucketDirectoryPath</t>
-  </si>
-  <si>
-    <t>DU_AutocorrectStorageBucketDirectoryPath</t>
-  </si>
-  <si>
-    <t>Path inside the Storage Bucket where the autocorrect file is stored. The asset value overrides the one from the "AutocorrectOcrMistakes" sheet</t>
-  </si>
-  <si>
-    <t>MinimumNumberOfRepetitions</t>
-  </si>
-  <si>
-    <t>DU_MinimumNumberOfRepetitions</t>
-  </si>
-  <si>
-    <t>The minimum number of times the value needs to be corrected in Action Center before the flow will start to autocorrect. The asset value overrides the one from the "AutocorrectOcrMistakes" sheet</t>
-  </si>
-  <si>
-    <t>AutocorrectionEnabled</t>
-  </si>
-  <si>
-    <t>DU_AutocorrectionEnabled</t>
-  </si>
-  <si>
-    <t>A flag that determines if autocorrection should be called or not. The asset value overrides the one from the "AutocorrectOcrMistakes" sheet</t>
-  </si>
-  <si>
-    <t>AutocorrectionFieldIdList</t>
-  </si>
-  <si>
-    <t>DU_AutocorrectionFieldIdList</t>
-  </si>
-  <si>
-    <t>A comma separated list of the taxonomy ids of the fields we want to enable autocorrection for. Has a corresponding asset that can be configured to overwrite this setting.</t>
-  </si>
-  <si>
-    <t>LogMessage_InvoicePostProcessing</t>
-  </si>
-  <si>
-    <t>Starting Invoice Post Processing</t>
-  </si>
-  <si>
-    <t>LogMessage_InvoicePostProcessing_DateFailure</t>
-  </si>
-  <si>
-    <t>Parsing the Date has failed!</t>
-  </si>
-  <si>
-    <t>LogMessage_InvoicePostProcessing_MandatoryFieldsFailure</t>
-  </si>
-  <si>
-    <t>One or more of the mandatory were missing!</t>
-  </si>
-  <si>
-    <t>LogMessage_InvoicePostProcessing_LineAmountFailureMath</t>
-  </si>
-  <si>
-    <t>Quantity * Unit-price is not equal to Line Amount!</t>
-  </si>
-  <si>
-    <t>LogMessage_InvoicePostProcessing_LineAmountFailureEmpty</t>
-  </si>
-  <si>
-    <t>Quantity or Unit-price is Empty!</t>
-  </si>
-  <si>
-    <t>LogMessage_InvoicePostProcessing_AlreadySetFalse</t>
-  </si>
-  <si>
-    <t>AutoExtraction is already set to false in a previous step. Skipping rest of checks.</t>
-  </si>
-  <si>
-    <t>LogMessage_InvoicePostProcessing_SubtotalFailure</t>
-  </si>
-  <si>
-    <t>Subtotal Failure with subtotal: {0} and net-amount {1}</t>
-  </si>
-  <si>
-    <t>LogMessage_InvoicePostProcessing_TotalFailure</t>
-  </si>
-  <si>
-    <t>Total Computation Failed!</t>
-  </si>
-  <si>
-    <t>LogMessage_InvoicePostProcessing_SubtotalPass</t>
-  </si>
-  <si>
-    <t>Subtotal Pass with subtotal: {0} and net-amount {1}</t>
-  </si>
-  <si>
-    <t>LogMessage_InvoicePostProcessing_ConfidenceFieldsFailure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">These are the fields that failed: </t>
-  </si>
-  <si>
-    <t>SubTotalAdditions</t>
-  </si>
-  <si>
-    <t>Tax Amount,Shipping Charges,Discount</t>
-  </si>
-  <si>
-    <t>Each field present in the list here, will be added to the subtotal to compute the total</t>
-  </si>
-  <si>
-    <t>MandatoryFields</t>
-  </si>
-  <si>
-    <t>Date,Invoice Number,PO Number,Total</t>
-  </si>
-  <si>
-    <t>These fields are mandatory. If they have not been extracted at all, the document will be sent for validation</t>
-  </si>
-  <si>
-    <t>MandatoryColumnFields</t>
-  </si>
-  <si>
-    <t>Quantity,Unit Price,Line Amount</t>
-  </si>
-  <si>
-    <t>These column fields are mandatory. If they have not been extracted at all, the document will be sent for validation</t>
-  </si>
-  <si>
-    <t>ConfidenceFields</t>
-  </si>
-  <si>
-    <t>Date,Shipping Address,Invoice Number,PO Number</t>
-  </si>
-  <si>
-    <t>List of fields which will be checked versus a specific confidence threshold. All new entries must have the "-Confidence" suffix</t>
-  </si>
-  <si>
-    <t>OtherConfidenceFields</t>
-  </si>
-  <si>
-    <t>Tax Amount,Net Amount,Discount,Shipping Charges,Billing Name,Total, Name, Vendor Address, Billing Address, Billing VAT Number, Payment Address, Vendor VAT Number, DueDate,Payment Terms</t>
-  </si>
-  <si>
-    <t>List of fields which will be checked versus a single confidence #:  Other-Confidence</t>
-  </si>
-  <si>
-    <t>Date-Confidence</t>
-  </si>
-  <si>
-    <t>Shipping Address-Confidence</t>
-  </si>
-  <si>
-    <t>Invoice Number-Confidence</t>
-  </si>
-  <si>
-    <t>PO Number-Confidence</t>
-  </si>
-  <si>
-    <t>other-Confidence</t>
-  </si>
-  <si>
-    <t>AutocorrectionLearningFile.json</t>
-  </si>
-  <si>
-    <t>Path inside the Storage Bucket where the autocorrect file is stored. Has a corresponding asset that can be configured to overwrite this setting.</t>
-  </si>
-  <si>
-    <t>The minimum number of times the value needs to be corrected in Action Center before the flow will start to autocorrect. Has a corresponding asset that can be configured to overwrite this setting.</t>
-  </si>
-  <si>
-    <t>A flag that determines if autocorrection should be called or not. Has a corresponding asset that can be configured to overwrite this setting.</t>
+    <t>MaxAttempts</t>
+  </si>
+  <si>
+    <t>OCR_API_Key</t>
+  </si>
+  <si>
+    <t>Google_GenAI_Endpoint</t>
+  </si>
+  <si>
+    <t>Gemini_API_Key</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -973,18 +755,11 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="238"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1022,8 +797,8 @@
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperłącze" xfId="1" builtinId="8"/>
@@ -2673,7 +2448,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z988"/>
+  <dimension ref="A1:Z991"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
@@ -2941,393 +2716,411 @@
         <v>127</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1">
+      <c r="C27" s="2"/>
+    </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>129</v>
-      </c>
-      <c r="B28" t="s">
-        <v>130</v>
-      </c>
+        <v>223</v>
+      </c>
+      <c r="B28">
+        <v>3</v>
+      </c>
+      <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>131</v>
-      </c>
-      <c r="B29" t="s">
-        <v>132</v>
-      </c>
+        <v>126</v>
+      </c>
+      <c r="B29" s="7">
+        <v>5.7870370370370373E-5</v>
+      </c>
+      <c r="C29" s="2"/>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B31" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
       <c r="A32" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B32" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A33" t="s">
-        <v>137</v>
-      </c>
-      <c r="B33" t="s">
-        <v>138</v>
-      </c>
-    </row>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="34" spans="1:2" ht="14.25" customHeight="1">
       <c r="A34" t="s">
-        <v>139</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>140</v>
+        <v>133</v>
+      </c>
+      <c r="B34" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="B35" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1">
       <c r="A36" t="s">
-        <v>143</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>144</v>
+        <v>137</v>
+      </c>
+      <c r="B36" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1">
       <c r="A37" t="s">
-        <v>145</v>
-      </c>
-      <c r="B37" t="s">
-        <v>146</v>
+        <v>139</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B38" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>149</v>
-      </c>
-      <c r="B39" t="s">
-        <v>150</v>
+        <v>143</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B40" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="B41" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="B42" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B43" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="B44" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
       <c r="A45" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B45" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A46" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>164</v>
+      <c r="A46" t="s">
+        <v>157</v>
+      </c>
+      <c r="B46" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="B47" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B48" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A49" t="s">
-        <v>169</v>
-      </c>
-      <c r="B49" t="s">
-        <v>170</v>
+      <c r="A49" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.25" customHeight="1">
       <c r="A50" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B50" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="14.25" customHeight="1">
       <c r="A51" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B51" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="14.25" customHeight="1">
       <c r="A52" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B52" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="14.25" customHeight="1">
       <c r="A53" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="B53" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="14.25" customHeight="1">
       <c r="A54" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B54" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="14.25" customHeight="1">
       <c r="A55" t="s">
+        <v>175</v>
+      </c>
+      <c r="B55" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A56" t="s">
+        <v>177</v>
+      </c>
+      <c r="B56" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A57" t="s">
+        <v>179</v>
+      </c>
+      <c r="B57" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A58" t="s">
         <v>181</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B58" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="56" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A56" s="2" t="s">
+    <row r="59" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A59" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B59" s="2" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="57" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A57" s="2" t="s">
+    <row r="60" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A60" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B60" s="2" t="s">
         <v>186</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="59" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A59" t="s">
-        <v>187</v>
-      </c>
-      <c r="B59" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A60" t="s">
-        <v>189</v>
-      </c>
-      <c r="B60" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="62" spans="1:2" ht="14.25" customHeight="1">
       <c r="A62" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B62" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="14.25" customHeight="1">
       <c r="A63" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B63" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A64" t="s">
-        <v>195</v>
-      </c>
-      <c r="B64" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" ht="14.25" customHeight="1"/>
+        <v>190</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="65" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A65" t="s">
+        <v>191</v>
+      </c>
+      <c r="B65" t="s">
+        <v>192</v>
+      </c>
+    </row>
     <row r="66" spans="1:2" ht="14.25" customHeight="1">
       <c r="A66" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B66" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="14.25" customHeight="1">
       <c r="A67" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B67" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A68" t="s">
-        <v>201</v>
-      </c>
-      <c r="B68" t="s">
-        <v>202</v>
-      </c>
-    </row>
+        <v>196</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="69" spans="1:2" ht="14.25" customHeight="1">
       <c r="A69" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="B69" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="14.25" customHeight="1">
       <c r="A70" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="B70" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="14.25" customHeight="1">
       <c r="A71" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B71" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="14.25" customHeight="1">
       <c r="A72" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B72" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" ht="14.25" customHeight="1"/>
+        <v>204</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A73" t="s">
+        <v>205</v>
+      </c>
+      <c r="B73" t="s">
+        <v>206</v>
+      </c>
+    </row>
     <row r="74" spans="1:2" ht="14.25" customHeight="1">
       <c r="A74" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B74" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="14.25" customHeight="1">
       <c r="A75" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="B75" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="77" spans="1:2" ht="14.25" customHeight="1">
       <c r="A77" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B77" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="79" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A79" t="s">
-        <v>217</v>
-      </c>
-      <c r="B79" t="s">
-        <v>218</v>
-      </c>
-    </row>
+        <v>212</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A78" t="s">
+        <v>213</v>
+      </c>
+      <c r="B78" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="80" spans="1:2" ht="14.25" customHeight="1">
       <c r="A80" t="s">
+        <v>215</v>
+      </c>
+      <c r="B80" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="82" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A82" t="s">
+        <v>217</v>
+      </c>
+      <c r="B82" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A83" t="s">
         <v>219</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B83" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="81" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A81" t="s">
+    <row r="84" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A84" t="s">
         <v>221</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B84" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="82" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="83" spans="1:2" ht="14.25" customHeight="1"/>
-    <row r="84" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="85" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="86" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="87" spans="1:2" ht="14.25" customHeight="1"/>
@@ -4232,6 +4025,9 @@
     <row r="986" ht="14.25" customHeight="1"/>
     <row r="987" ht="14.25" customHeight="1"/>
     <row r="988" ht="14.25" customHeight="1"/>
+    <row r="989" ht="14.25" customHeight="1"/>
+    <row r="990" ht="14.25" customHeight="1"/>
+    <row r="991" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4239,12 +4035,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z1000"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A750E08D-D02E-430F-882B-99071203194A}">
+  <dimension ref="A1:Z980"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
+    <col min="2" max="2" width="40.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="60.28515625" customWidth="1"/>
     <col min="4" max="26" width="65.42578125" customWidth="1"/>
   </cols>
@@ -4287,209 +4083,56 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B2" t="s">
         <v>224</v>
       </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="3" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A3" s="8" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="3" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="B3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A4" s="8" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A4" t="s">
-        <v>86</v>
-      </c>
       <c r="B4" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A6" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A8" t="s">
-        <v>101</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="D8" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A9" t="s">
-        <v>103</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="D9" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A10" t="s">
-        <v>105</v>
-      </c>
-      <c r="B10" t="s">
-        <v>234</v>
-      </c>
-      <c r="D10" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" t="s">
-        <v>107</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="D11" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A12" t="s">
-        <v>109</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="D12" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A13" t="s">
-        <v>112</v>
-      </c>
-      <c r="B13" t="s">
-        <v>240</v>
-      </c>
-      <c r="D13" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A14" t="s">
-        <v>93</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
+        <v>226</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A16" t="s">
-        <v>243</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="D16" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A17" t="s">
-        <v>246</v>
-      </c>
-      <c r="B17" t="s">
-        <v>247</v>
-      </c>
-      <c r="D17" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A18" t="s">
-        <v>249</v>
-      </c>
-      <c r="B18" t="s">
-        <v>250</v>
-      </c>
-      <c r="D18" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A19" t="s">
-        <v>252</v>
-      </c>
-      <c r="B19" t="s">
-        <v>253</v>
-      </c>
-      <c r="D19" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="21" spans="1:4" ht="14.25" customHeight="1">
-      <c r="A21" t="s">
-        <v>98</v>
-      </c>
-      <c r="B21" t="s">
-        <v>98</v>
-      </c>
-      <c r="D21" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="23" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="24" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="25" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="26" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="27" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="28" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="29" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="30" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="31" spans="1:4" ht="14.25" customHeight="1"/>
-    <row r="32" spans="1:4" ht="14.25" customHeight="1"/>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="17" ht="14.25" customHeight="1"/>
+    <row r="18" ht="14.25" customHeight="1"/>
+    <row r="19" ht="14.25" customHeight="1"/>
+    <row r="20" ht="14.25" customHeight="1"/>
+    <row r="21" ht="14.25" customHeight="1"/>
+    <row r="22" ht="14.25" customHeight="1"/>
+    <row r="23" ht="14.25" customHeight="1"/>
+    <row r="24" ht="14.25" customHeight="1"/>
+    <row r="25" ht="14.25" customHeight="1"/>
+    <row r="26" ht="14.25" customHeight="1"/>
+    <row r="27" ht="14.25" customHeight="1"/>
+    <row r="28" ht="14.25" customHeight="1"/>
+    <row r="29" ht="14.25" customHeight="1"/>
+    <row r="30" ht="14.25" customHeight="1"/>
+    <row r="31" ht="14.25" customHeight="1"/>
+    <row r="32" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>
@@ -5438,1380 +5081,6 @@
     <row r="978" ht="14.25" customHeight="1"/>
     <row r="979" ht="14.25" customHeight="1"/>
     <row r="980" ht="14.25" customHeight="1"/>
-    <row r="981" ht="14.25" customHeight="1"/>
-    <row r="982" ht="14.25" customHeight="1"/>
-    <row r="983" ht="14.25" customHeight="1"/>
-    <row r="984" ht="14.25" customHeight="1"/>
-    <row r="985" ht="14.25" customHeight="1"/>
-    <row r="986" ht="14.25" customHeight="1"/>
-    <row r="987" ht="14.25" customHeight="1"/>
-    <row r="988" ht="14.25" customHeight="1"/>
-    <row r="989" ht="14.25" customHeight="1"/>
-    <row r="990" ht="14.25" customHeight="1"/>
-    <row r="991" ht="14.25" customHeight="1"/>
-    <row r="992" ht="14.25" customHeight="1"/>
-    <row r="993" ht="14.25" customHeight="1"/>
-    <row r="994" ht="14.25" customHeight="1"/>
-    <row r="995" ht="14.25" customHeight="1"/>
-    <row r="996" ht="14.25" customHeight="1"/>
-    <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
-    <row r="999" ht="14.25" customHeight="1"/>
-    <row r="1000" ht="14.25" customHeight="1"/>
-  </sheetData>
-  <phoneticPr fontId="2"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92A4CE3F-370D-498E-8CEC-17EC0E626FC8}">
-  <dimension ref="A1:C25"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="57.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="72.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="115" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>255</v>
-      </c>
-      <c r="B3" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>257</v>
-      </c>
-      <c r="B4" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>259</v>
-      </c>
-      <c r="B5" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>261</v>
-      </c>
-      <c r="B6" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>263</v>
-      </c>
-      <c r="B7" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>265</v>
-      </c>
-      <c r="B8" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>267</v>
-      </c>
-      <c r="B9" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>269</v>
-      </c>
-      <c r="B10" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>271</v>
-      </c>
-      <c r="B11" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
-        <v>273</v>
-      </c>
-      <c r="B13" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3">
-      <c r="A15" t="s">
-        <v>275</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>276</v>
-      </c>
-      <c r="C15" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3">
-      <c r="A16" t="s">
-        <v>278</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="C16" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17" t="s">
-        <v>281</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>282</v>
-      </c>
-      <c r="C17" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="A18" t="s">
-        <v>284</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>285</v>
-      </c>
-      <c r="C18" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
-        <v>287</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>288</v>
-      </c>
-      <c r="C19" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3">
-      <c r="A21" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="B21">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
-      <c r="A22" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="B22">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
-      <c r="A23" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="B23">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="B24">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3">
-      <c r="A25" t="s">
-        <v>294</v>
-      </c>
-      <c r="B25">
-        <v>45</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5740500-B5EB-4696-A4C0-ED7892074369}">
-  <dimension ref="A1:Z1005"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="43.85546875" customWidth="1"/>
-    <col min="2" max="2" width="70.140625" customWidth="1"/>
-    <col min="3" max="3" width="166" bestFit="1" customWidth="1"/>
-    <col min="4" max="26" width="8.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A1" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
-      <c r="N1" s="8"/>
-      <c r="O1" s="8"/>
-      <c r="P1" s="8"/>
-      <c r="Q1" s="8"/>
-      <c r="R1" s="8"/>
-      <c r="S1" s="8"/>
-      <c r="T1" s="8"/>
-      <c r="U1" s="8"/>
-      <c r="V1" s="8"/>
-      <c r="W1" s="8"/>
-      <c r="X1" s="8"/>
-      <c r="Y1" s="8"/>
-      <c r="Z1" s="8"/>
-    </row>
-    <row r="2" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A2" s="8"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8"/>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="8"/>
-      <c r="S2" s="8"/>
-      <c r="T2" s="8"/>
-      <c r="U2" s="8"/>
-      <c r="V2" s="8"/>
-      <c r="W2" s="8"/>
-      <c r="X2" s="8"/>
-      <c r="Y2" s="8"/>
-      <c r="Z2" s="8"/>
-    </row>
-    <row r="3" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A3" t="s">
-        <v>243</v>
-      </c>
-      <c r="B3" t="s">
-        <v>295</v>
-      </c>
-      <c r="C3" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A5" t="s">
-        <v>246</v>
-      </c>
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A6" t="s">
-        <v>249</v>
-      </c>
-      <c r="B6" t="b">
-        <v>0</v>
-      </c>
-      <c r="C6" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" t="s">
-        <v>252</v>
-      </c>
-      <c r="C7" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A16" s="2"/>
-      <c r="B16" s="6"/>
-      <c r="C16" s="2"/>
-    </row>
-    <row r="17" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A17" s="2"/>
-      <c r="B17" s="6"/>
-      <c r="C17" s="2"/>
-    </row>
-    <row r="18" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A18" s="2"/>
-      <c r="B18" s="6"/>
-      <c r="C18" s="2"/>
-    </row>
-    <row r="19" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A19" s="2"/>
-      <c r="B19" s="6"/>
-      <c r="C19" s="2"/>
-    </row>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A20" s="2"/>
-      <c r="B20" s="6"/>
-      <c r="C20" s="2"/>
-    </row>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1">
-      <c r="C21" s="2"/>
-    </row>
-    <row r="22" spans="1:3" ht="14.25" customHeight="1">
-      <c r="C22" s="2"/>
-    </row>
-    <row r="23" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B23" s="2"/>
-    </row>
-    <row r="24" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B24" s="2"/>
-    </row>
-    <row r="25" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B25" s="2"/>
-    </row>
-    <row r="26" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="27" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B27" s="2"/>
-    </row>
-    <row r="28" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="29" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B29" s="2"/>
-    </row>
-    <row r="30" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="32" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="33" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="34" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="35" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="36" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="37" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="38" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="39" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="40" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="41" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="42" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="43" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="44" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="45" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="46" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="47" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="48" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="49" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="50" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="51" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="52" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="53" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="54" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="55" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="56" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="57" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="58" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="59" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="60" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="61" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="62" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="63" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="64" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="65" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="66" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="67" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="68" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="69" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="70" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="71" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="72" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="73" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="74" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="75" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="76" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="77" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="78" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="79" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="80" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="81" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="82" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="83" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="84" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="85" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="86" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="87" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="88" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="89" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="90" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="91" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="92" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="93" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="94" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="95" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="96" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="97" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="98" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="99" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="100" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="101" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="102" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="103" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="104" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="105" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="106" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="107" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="108" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="109" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="110" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="111" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="112" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="113" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="114" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="115" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="116" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="117" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="118" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="119" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="120" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="121" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="122" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="123" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="124" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="125" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="126" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="127" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="128" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="129" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="130" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="131" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="132" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="133" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="134" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="135" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="136" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="137" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="138" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="139" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="140" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="141" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="142" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="143" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="144" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="145" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="146" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="147" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="148" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="149" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="150" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="151" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="152" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="153" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="154" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="155" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="156" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="157" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="158" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="159" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="160" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="161" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="162" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="163" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="164" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="165" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="166" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="167" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="168" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="169" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="170" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="171" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="172" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="173" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="174" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="175" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="176" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="177" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="178" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="179" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="180" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="181" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="182" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="183" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="184" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="185" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="186" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="187" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="188" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="189" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="190" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="191" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="192" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="193" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="194" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="195" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="196" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="197" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="198" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="199" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="200" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="201" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="202" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="203" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="204" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="205" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="206" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="207" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="208" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="209" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="210" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="211" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="212" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="213" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="214" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="215" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="216" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="217" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="218" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="219" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="220" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="221" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="222" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="223" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="224" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="225" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="226" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="227" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="228" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="229" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="230" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="231" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="232" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="233" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="234" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="235" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="236" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="237" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="238" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="239" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="240" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="241" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="242" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="243" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="244" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="245" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="246" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="247" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="248" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="249" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="250" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="251" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="252" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="253" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="254" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="255" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="256" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="257" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="258" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="259" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="260" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="261" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="262" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="263" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="264" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="265" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="266" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="267" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="268" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="269" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="270" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="271" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="272" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="273" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="274" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="275" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="276" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="277" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="278" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="279" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="280" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="281" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="282" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="283" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="284" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="285" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="286" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="287" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="288" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="289" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="290" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="291" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="292" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="293" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="294" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="295" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="296" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="297" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="298" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="299" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="300" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="301" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="302" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="303" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="304" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="305" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="306" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="307" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="308" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="309" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="310" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="311" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="312" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="313" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="314" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="315" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="316" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="317" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="318" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="319" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="320" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="321" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="322" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="323" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="324" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="325" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="326" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="327" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="328" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="329" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="330" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="331" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="332" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="333" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="334" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="335" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="336" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="337" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="338" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="339" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="340" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="341" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="342" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="343" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="344" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="345" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="346" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="347" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="348" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="349" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="350" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="351" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="352" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="353" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="354" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="355" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="356" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="357" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="358" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="359" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="360" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="361" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="362" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="363" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="364" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="365" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="366" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="367" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="368" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="369" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="370" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="371" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="372" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="373" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="374" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="375" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="376" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="377" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="378" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="379" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="380" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="381" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="382" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="383" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="384" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="385" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="386" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="387" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="388" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="389" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="390" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="391" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="392" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="393" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="394" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="395" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="396" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="397" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="398" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="399" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="400" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="401" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="402" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="403" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="404" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="405" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="406" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="407" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="408" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="409" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="410" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="411" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="412" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="413" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="414" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="415" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="416" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="417" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="418" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="419" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="420" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="421" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="422" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="423" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="424" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="425" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="426" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="427" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="428" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="429" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="430" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="431" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="432" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="433" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="434" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="435" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="436" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="437" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="438" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="439" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="440" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="441" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="442" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="443" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="444" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="445" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="446" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="447" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="448" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="449" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="450" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="451" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="452" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="453" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="454" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="455" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="456" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="457" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="458" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="459" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="460" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="461" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="462" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="463" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="464" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="465" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="466" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="467" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="468" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="469" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="470" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="471" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="472" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="473" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="474" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="475" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="476" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="477" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="478" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="479" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="480" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="481" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="482" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="483" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="484" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="485" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="486" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="487" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="488" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="489" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="490" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="491" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="492" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="493" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="494" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="495" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="496" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="497" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="498" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="499" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="500" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="501" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="502" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="503" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="504" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="505" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="506" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="507" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="508" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="509" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="510" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="511" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="512" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="513" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="514" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="515" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="516" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="517" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="518" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="519" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="520" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="521" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="522" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="523" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="524" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="525" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="526" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="527" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="528" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="529" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="530" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="531" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="532" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="533" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="534" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="535" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="536" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="537" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="538" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="539" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="540" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="541" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="542" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="543" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="544" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="545" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="546" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="547" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="548" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="549" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="550" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="551" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="552" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="553" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="554" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="555" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="556" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="557" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="558" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="559" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="560" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="561" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="562" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="563" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="564" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="565" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="566" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="567" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="568" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="569" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="570" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="571" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="572" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="573" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="574" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="575" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="576" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="577" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="578" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="579" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="580" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="581" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="582" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="583" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="584" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="585" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="586" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="587" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="588" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="589" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="590" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="591" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="592" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="593" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="594" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="595" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="596" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="597" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="598" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="599" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="600" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="601" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="602" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="603" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="604" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="605" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="606" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="607" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="608" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="609" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="610" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="611" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="612" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="613" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="614" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="615" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="616" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="617" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="618" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="619" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="620" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="621" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="622" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="623" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="624" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="625" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="626" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="627" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="628" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="629" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="630" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="631" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="632" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="633" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="634" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="635" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="636" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="637" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="638" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="639" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="640" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="641" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="642" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="643" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="644" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="645" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="646" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="647" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="648" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="649" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="650" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="651" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="652" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="653" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="654" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="655" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="656" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="657" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="658" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="659" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="660" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="661" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="662" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="663" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="664" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="665" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="666" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="667" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="668" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="669" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="670" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="671" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="672" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="673" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="674" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="675" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="676" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="677" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="678" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="679" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="680" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="681" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="682" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="683" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="684" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="685" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="686" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="687" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="688" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="689" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="690" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="691" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="692" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="693" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="694" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="695" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="696" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="697" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="698" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="699" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="700" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="701" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="702" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="703" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="704" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="705" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="706" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="707" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="708" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="709" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="710" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="711" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="712" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="713" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="714" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="715" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="716" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="717" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="718" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="719" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="720" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="721" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="722" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="723" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="724" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="725" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="726" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="727" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="728" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="729" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="730" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="731" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="732" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="733" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="734" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="735" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="736" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="737" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="738" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="739" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="740" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="741" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="742" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="743" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="744" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="745" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="746" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="747" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="748" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="749" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="750" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="751" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="752" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="753" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="754" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="755" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="756" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="757" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="758" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="759" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="760" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="761" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="762" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="763" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="764" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="765" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="766" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="767" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="768" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="769" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="770" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="771" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="772" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="773" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="774" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="775" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="776" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="777" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="778" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="779" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="780" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="781" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="782" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="783" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="784" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="785" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="786" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="787" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="788" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="789" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="790" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="791" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="792" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="793" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="794" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="795" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="796" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="797" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="798" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="799" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="800" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="801" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="802" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="803" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="804" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="805" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="806" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="807" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="808" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="809" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="810" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="811" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="812" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="813" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="814" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="815" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="816" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="817" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="818" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="819" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="820" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="821" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="822" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="823" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="824" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="825" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="826" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="827" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="828" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="829" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="830" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="831" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="832" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="833" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="834" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="835" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="836" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="837" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="838" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="839" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="840" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="841" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="842" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="843" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="844" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="845" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="846" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="847" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="848" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="849" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="850" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="851" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="852" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="853" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="854" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="855" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="856" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="857" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="858" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="859" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="860" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="861" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="862" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="863" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="864" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="865" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="866" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="867" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="868" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="869" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="870" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="871" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="872" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="873" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="874" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="875" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="876" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="877" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="878" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="879" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="880" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="881" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="882" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="883" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="884" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="885" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="886" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="887" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="888" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="889" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="890" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="891" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="892" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="893" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="894" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="895" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="896" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="897" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="898" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="899" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="900" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="901" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="902" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="903" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="904" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="905" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="906" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="907" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="908" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="909" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="910" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="911" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="912" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="913" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="914" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="915" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="916" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="917" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="918" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="919" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="920" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="921" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="922" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="923" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="924" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="925" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="926" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="927" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="928" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="929" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="930" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="931" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="932" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="933" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="934" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="935" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="936" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="937" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="938" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="939" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="940" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="941" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="942" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="943" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="944" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="945" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="946" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="947" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="948" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="949" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="950" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="951" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="952" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="953" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="954" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="955" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="956" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="957" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="958" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="959" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="960" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="961" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="962" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="963" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="964" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="965" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="966" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="967" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="968" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="969" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="970" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="971" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="972" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="973" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="974" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="975" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="976" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="977" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="978" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="979" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="980" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="981" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="982" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="983" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="984" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="985" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="986" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="987" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="988" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="989" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="990" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="991" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="992" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="993" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="994" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="995" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="996" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="997" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="998" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="999" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="1000" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="1001" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="1002" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="1003" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="1004" customFormat="1" ht="14.25" customHeight="1"/>
-    <row r="1005" customFormat="1" ht="14.25" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Change DU to Google Gemini
</commit_message>
<xml_diff>
--- a/RegEx Document Processing Demo/Data/Config.xlsx
+++ b/RegEx Document Processing Demo/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci\Documents\UiPath\REPO\RegEx Document Processing Demo\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51AFD3D-FE7D-43D1-9E96-C1875C35E69A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D02D1E-8281-489F-8D39-DE2D316FA211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="230">
   <si>
     <t>Name</t>
   </si>
@@ -156,12 +156,6 @@
     <t xml:space="preserve">The maximum number of consecutive system exceptions was reached. </t>
   </si>
   <si>
-    <t>RegEx Document Processing Demo</t>
-  </si>
-  <si>
-    <t>RegEx_Document_Processing_Demo</t>
-  </si>
-  <si>
     <t>InputFolder</t>
   </si>
   <si>
@@ -706,6 +700,21 @@
   </si>
   <si>
     <t>Gemini_API_Key</t>
+  </si>
+  <si>
+    <t>Document_Processing</t>
+  </si>
+  <si>
+    <t>Document_Processing_Demo</t>
+  </si>
+  <si>
+    <t>Document Processing Demo</t>
+  </si>
+  <si>
+    <t>CacheFolder</t>
+  </si>
+  <si>
+    <t>C:\RPA\Cache</t>
   </si>
 </sst>
 </file>
@@ -1114,7 +1123,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z998"/>
+  <dimension ref="A1:Z999"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -1162,7 +1171,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>44</v>
+        <v>226</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>21</v>
@@ -1172,7 +1181,9 @@
       <c r="A3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" s="2" t="s">
+        <v>225</v>
+      </c>
       <c r="C3" s="4" t="s">
         <v>31</v>
       </c>
@@ -1183,7 +1194,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>43</v>
+        <v>227</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>22</v>
@@ -1192,48 +1203,48 @@
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" t="s">
-        <v>59</v>
-      </c>
-      <c r="B11" t="s">
-        <v>54</v>
-      </c>
-    </row>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" t="s">
+        <v>228</v>
+      </c>
+      <c r="B10" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B13" t="s">
         <v>51</v>
@@ -1241,251 +1252,258 @@
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B14" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B15" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A17" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="19" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A21" t="s">
+        <v>63</v>
+      </c>
+      <c r="B21" t="s">
         <v>64</v>
       </c>
-      <c r="B16" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="18" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A18" t="s">
-        <v>56</v>
-      </c>
-      <c r="B18" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A20" t="s">
+      <c r="C21" t="s">
         <v>65</v>
       </c>
-      <c r="B20" t="s">
-        <v>66</v>
-      </c>
-      <c r="C20" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="22" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A22" t="s">
-        <v>68</v>
-      </c>
-      <c r="B22" t="s">
-        <v>69</v>
-      </c>
-      <c r="C22" t="s">
-        <v>70</v>
-      </c>
-    </row>
+    </row>
+    <row r="22" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
       <c r="A23" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B23" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C23" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="B24" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C24" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1">
       <c r="A25" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B25" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C25" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
       <c r="A26" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" t="s">
+        <v>76</v>
+      </c>
+      <c r="C26" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A27" t="s">
+        <v>78</v>
+      </c>
+      <c r="B27" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" t="s">
         <v>80</v>
       </c>
-      <c r="B26" t="s">
-        <v>81</v>
-      </c>
-      <c r="C26" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="28" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A28" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
+    </row>
+    <row r="28" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="29" spans="1:3" ht="14.25" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A33" s="2"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="2"/>
+    </row>
+    <row r="34" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A34" t="s">
         <v>91</v>
       </c>
-      <c r="B31" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="C31" s="2" t="s">
+      <c r="B34">
+        <v>0.5</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A32" s="2"/>
-      <c r="B32" s="6"/>
-      <c r="C32" s="2"/>
-    </row>
-    <row r="33" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A33" t="s">
+    <row r="35" spans="1:3" ht="14.25" customHeight="1">
+      <c r="C35" s="2"/>
+    </row>
+    <row r="36" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A36" t="s">
         <v>93</v>
       </c>
-      <c r="B33">
-        <v>0.5</v>
-      </c>
-      <c r="C33" s="2" t="s">
+      <c r="B36" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" ht="14.25" customHeight="1">
-      <c r="C34" s="2"/>
-    </row>
-    <row r="35" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A35" t="s">
+      <c r="C36" t="s">
         <v>95</v>
       </c>
-      <c r="B35" s="2" t="s">
+    </row>
+    <row r="37" spans="1:3" ht="14.25" customHeight="1">
+      <c r="B37" s="2"/>
+    </row>
+    <row r="38" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A38" t="s">
         <v>96</v>
       </c>
-      <c r="C35" t="s">
+      <c r="B38" s="2" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B36" s="2"/>
-    </row>
-    <row r="37" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A37" t="s">
+      <c r="C38" t="s">
         <v>98</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C37" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B38" s="2"/>
     </row>
     <row r="39" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A39" t="s">
-        <v>101</v>
-      </c>
       <c r="B39" s="2"/>
-      <c r="C39" t="s">
-        <v>102</v>
-      </c>
     </row>
     <row r="40" spans="1:3" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>103</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="B40" s="2"/>
       <c r="C40" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>105</v>
-      </c>
-      <c r="B41" s="2"/>
+        <v>101</v>
+      </c>
       <c r="C41" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>107</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="B42" s="2"/>
       <c r="C42" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>109</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="C43" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>112</v>
+        <v>107</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>108</v>
       </c>
       <c r="C44" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" ht="14.25" customHeight="1"/>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A45" t="s">
+        <v>110</v>
+      </c>
+      <c r="C45" t="s">
+        <v>111</v>
+      </c>
+    </row>
     <row r="46" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="47" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="48" spans="1:3" ht="14.25" customHeight="1"/>
@@ -2439,6 +2457,7 @@
     <row r="996" ht="14.25" customHeight="1"/>
     <row r="997" ht="14.25" customHeight="1"/>
     <row r="998" ht="14.25" customHeight="1"/>
+    <row r="999" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2630,90 +2649,90 @@
     <row r="18" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B19">
         <v>3</v>
       </c>
       <c r="C19" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B20">
         <v>3</v>
       </c>
       <c r="C20" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B21">
         <v>3</v>
       </c>
       <c r="C21" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B22">
         <v>3</v>
       </c>
       <c r="C22" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
       <c r="A23" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B23">
         <v>99999</v>
       </c>
       <c r="C23" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B24">
         <v>30</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1">
       <c r="A25" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B25">
         <v>30</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
       <c r="A26" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B26">
         <v>1</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
@@ -2721,7 +2740,7 @@
     </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B28">
         <v>3</v>
@@ -2730,7 +2749,7 @@
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B29" s="7">
         <v>5.7870370370370373E-5</v>
@@ -2740,385 +2759,385 @@
     <row r="30" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B31" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
       <c r="A32" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B32" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="34" spans="1:2" ht="14.25" customHeight="1">
       <c r="A34" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B34" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B35" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1">
       <c r="A36" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B36" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="14.25" customHeight="1">
       <c r="A37" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="14.25" customHeight="1">
       <c r="A38" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B38" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="14.25" customHeight="1">
       <c r="A39" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="14.25" customHeight="1">
       <c r="A40" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B40" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B41" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B42" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B43" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B44" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="14.25" customHeight="1">
       <c r="A45" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B45" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="14.25" customHeight="1">
       <c r="A46" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B46" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="14.25" customHeight="1">
       <c r="A47" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B47" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="14.25" customHeight="1">
       <c r="A48" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B48" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="14.25" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="14.25" customHeight="1">
       <c r="A50" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B50" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="14.25" customHeight="1">
       <c r="A51" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B51" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="14.25" customHeight="1">
       <c r="A52" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B52" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="14.25" customHeight="1">
       <c r="A53" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B53" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="14.25" customHeight="1">
       <c r="A54" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B54" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="14.25" customHeight="1">
       <c r="A55" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B55" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="14.25" customHeight="1">
       <c r="A56" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B56" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="14.25" customHeight="1">
       <c r="A57" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B57" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="14.25" customHeight="1">
       <c r="A58" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B58" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="14.25" customHeight="1">
       <c r="A59" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="14.25" customHeight="1">
       <c r="A60" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="62" spans="1:2" ht="14.25" customHeight="1">
       <c r="A62" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B62" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="14.25" customHeight="1">
       <c r="A63" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B63" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="65" spans="1:2" ht="14.25" customHeight="1">
       <c r="A65" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B65" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="14.25" customHeight="1">
       <c r="A66" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B66" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="14.25" customHeight="1">
       <c r="A67" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B67" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="69" spans="1:2" ht="14.25" customHeight="1">
       <c r="A69" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B69" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="14.25" customHeight="1">
       <c r="A70" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B70" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="14.25" customHeight="1">
       <c r="A71" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B71" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="14.25" customHeight="1">
       <c r="A72" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B72" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="14.25" customHeight="1">
       <c r="A73" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B73" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="14.25" customHeight="1">
       <c r="A74" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B74" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="14.25" customHeight="1">
       <c r="A75" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B75" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="77" spans="1:2" ht="14.25" customHeight="1">
       <c r="A77" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B77" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="14.25" customHeight="1">
       <c r="A78" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B78" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="80" spans="1:2" ht="14.25" customHeight="1">
       <c r="A80" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B80" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="82" spans="1:2" ht="14.25" customHeight="1">
       <c r="A82" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B82" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="14.25" customHeight="1">
       <c r="A83" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B83" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="14.25" customHeight="1">
       <c r="A84" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B84" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="14.25" customHeight="1"/>
@@ -4083,26 +4102,35 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B2" t="s">
-        <v>224</v>
+        <v>222</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" s="8" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B3" t="s">
+        <v>223</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
       <c r="A4" s="8" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B4" t="s">
-        <v>226</v>
+        <v>224</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
add currency extraction to regex workflow
</commit_message>
<xml_diff>
--- a/RegEx Document Processing Demo/Data/Config.xlsx
+++ b/RegEx Document Processing Demo/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci\Documents\UiPath\REPO\RegEx Document Processing Demo\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D02D1E-8281-489F-8D39-DE2D316FA211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BFD0406-05B4-4358-B9BA-D9B91674DFCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="232">
   <si>
     <t>Name</t>
   </si>
@@ -715,6 +715,12 @@
   </si>
   <si>
     <t>C:\RPA\Cache</t>
+  </si>
+  <si>
+    <t>RegEx_Header_Currency</t>
+  </si>
+  <si>
+    <t>(?&lt;=Total:)\s?.(?=\d{1})</t>
   </si>
 </sst>
 </file>
@@ -1123,7 +1129,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z999"/>
+  <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -1268,243 +1274,250 @@
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>61</v>
+        <v>230</v>
       </c>
       <c r="B16" t="s">
-        <v>56</v>
+        <v>231</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1">
       <c r="A17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A18" t="s">
         <v>62</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="19" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A19" t="s">
+    <row r="19" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A20" t="s">
         <v>54</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B20" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A21" t="s">
+    <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="22" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A22" t="s">
         <v>63</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B22" t="s">
         <v>64</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C22" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="23" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A23" t="s">
-        <v>66</v>
-      </c>
-      <c r="B23" t="s">
-        <v>67</v>
-      </c>
-      <c r="C23" t="s">
-        <v>68</v>
-      </c>
-    </row>
+    <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B24" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C24" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1">
       <c r="A25" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B25" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C25" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C26" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
       <c r="A27" t="s">
+        <v>75</v>
+      </c>
+      <c r="B27" t="s">
+        <v>76</v>
+      </c>
+      <c r="C27" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A28" t="s">
         <v>78</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B28" t="s">
         <v>79</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C28" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="29" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A29" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
+    <row r="29" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>82</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>87</v>
       </c>
       <c r="C32" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A33" s="2"/>
-      <c r="B33" s="6"/>
-      <c r="C33" s="2"/>
-    </row>
     <row r="34" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A34" t="s">
+      <c r="A34" s="2"/>
+      <c r="B34" s="6"/>
+      <c r="C34" s="2"/>
+    </row>
+    <row r="35" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A35" t="s">
         <v>91</v>
       </c>
-      <c r="B34">
+      <c r="B35">
         <v>0.5</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="14.25" customHeight="1">
-      <c r="C35" s="2"/>
-    </row>
     <row r="36" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A36" t="s">
+      <c r="C36" s="2"/>
+    </row>
+    <row r="37" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A37" t="s">
         <v>93</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B37" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C37" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B37" s="2"/>
-    </row>
     <row r="38" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A38" t="s">
+      <c r="B38" s="2"/>
+    </row>
+    <row r="39" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A39" t="s">
         <v>96</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B39" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C39" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B39" s="2"/>
-    </row>
     <row r="40" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A40" t="s">
-        <v>99</v>
-      </c>
       <c r="B40" s="2"/>
-      <c r="C40" t="s">
-        <v>100</v>
-      </c>
     </row>
     <row r="41" spans="1:3" ht="14.25" customHeight="1">
       <c r="A41" t="s">
-        <v>101</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="B41" s="2"/>
       <c r="C41" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="14.25" customHeight="1">
       <c r="A42" t="s">
-        <v>103</v>
-      </c>
-      <c r="B42" s="2"/>
+        <v>101</v>
+      </c>
       <c r="C42" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>105</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="B43" s="2"/>
       <c r="C43" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="14.25" customHeight="1">
       <c r="A44" t="s">
-        <v>107</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C44" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="14.25" customHeight="1">
       <c r="A45" t="s">
+        <v>107</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C45" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A46" t="s">
         <v>110</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C46" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="47" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="48" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="49" ht="14.25" customHeight="1"/>
@@ -2458,6 +2471,7 @@
     <row r="997" ht="14.25" customHeight="1"/>
     <row r="998" ht="14.25" customHeight="1"/>
     <row r="999" ht="14.25" customHeight="1"/>
+    <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated the ai prompts
</commit_message>
<xml_diff>
--- a/RegEx Document Processing Demo/Data/Config.xlsx
+++ b/RegEx Document Processing Demo/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci\Documents\UiPath\REPO\RegEx Document Processing Demo\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BFD0406-05B4-4358-B9BA-D9B91674DFCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C926F8FA-4B02-4514-8AC4-7FF9E6934727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -717,10 +717,10 @@
     <t>C:\RPA\Cache</t>
   </si>
   <si>
-    <t>RegEx_Header_Currency</t>
-  </si>
-  <si>
     <t>(?&lt;=Total:)\s?.(?=\d{1})</t>
+  </si>
+  <si>
+    <t>RegEx_Footer_Currency</t>
   </si>
 </sst>
 </file>
@@ -1274,10 +1274,10 @@
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
+        <v>231</v>
+      </c>
+      <c r="B16" t="s">
         <v>230</v>
-      </c>
-      <c r="B16" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1">

</xml_diff>

<commit_message>
Finished the validation flow
</commit_message>
<xml_diff>
--- a/RegEx Document Processing Demo/Data/Config.xlsx
+++ b/RegEx Document Processing Demo/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci\Documents\UiPath\REPO\RegEx Document Processing Demo\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41427B64-97C9-4235-A713-CB5E21EBB255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C1CABCF-7E43-488A-98BF-3B47D5EB03CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="193">
   <si>
     <t>Name</t>
   </si>
@@ -592,6 +592,18 @@
   </si>
   <si>
     <t>number,date,vendor,amount,currency</t>
+  </si>
+  <si>
+    <t>AcceptedCurrencySymbols</t>
+  </si>
+  <si>
+    <t>$€£</t>
+  </si>
+  <si>
+    <t>ValidationRulesetVersion</t>
+  </si>
+  <si>
+    <t>1.0</t>
   </si>
 </sst>
 </file>
@@ -1191,8 +1203,22 @@
         <v>188</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="27" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="26" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A26" t="s">
+        <v>189</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A27" t="s">
+        <v>191</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="29" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="30" spans="1:3" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Added processing meta data string
</commit_message>
<xml_diff>
--- a/RegEx Document Processing Demo/Data/Config.xlsx
+++ b/RegEx Document Processing Demo/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci\Documents\UiPath\REPO\RegEx Document Processing Demo\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C1CABCF-7E43-488A-98BF-3B47D5EB03CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A161CC40-65E1-4A0D-84BB-F52B740B974C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="29580" yWindow="780" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="195">
   <si>
     <t>Name</t>
   </si>
@@ -604,6 +604,12 @@
   </si>
   <si>
     <t>1.0</t>
+  </si>
+  <si>
+    <t>PipelineVersion</t>
+  </si>
+  <si>
+    <t>1.0.0</t>
   </si>
 </sst>
 </file>
@@ -988,7 +994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z979"/>
+  <dimension ref="A1:Z980"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -1193,33 +1199,41 @@
       <c r="C23" s="2"/>
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B24" s="2"/>
+      <c r="A24" t="s">
+        <v>193</v>
+      </c>
+      <c r="B24" t="s">
+        <v>194</v>
+      </c>
+      <c r="C24" s="2"/>
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A25" t="s">
-        <v>187</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>188</v>
-      </c>
+      <c r="B25" s="2"/>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
       <c r="A26" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
       <c r="A27" t="s">
+        <v>189</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A28" t="s">
         <v>191</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B28" s="2" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="29" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="30" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="31" spans="1:3" ht="14.25" customHeight="1"/>
@@ -2171,6 +2185,7 @@
     <row r="977" ht="14.25" customHeight="1"/>
     <row r="978" ht="14.25" customHeight="1"/>
     <row r="979" ht="14.25" customHeight="1"/>
+    <row r="980" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Finished full document processing and validation with output separation
</commit_message>
<xml_diff>
--- a/RegEx Document Processing Demo/Data/Config.xlsx
+++ b/RegEx Document Processing Demo/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci\Documents\UiPath\REPO\RegEx Document Processing Demo\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E6C6AD8-79BA-482E-A9F2-C3F01B1DF028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{693ECC60-7177-48A4-9950-B6DAA71CA616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="203">
   <si>
     <t>Name</t>
   </si>
@@ -622,6 +622,18 @@
   </si>
   <si>
     <t>number,date,vendor,amount,currency,discount,shipping</t>
+  </si>
+  <si>
+    <t>OutputFolder_Valid</t>
+  </si>
+  <si>
+    <t>OutputFolder_Invalid</t>
+  </si>
+  <si>
+    <t>Data\Output\Valid</t>
+  </si>
+  <si>
+    <t>Data\Output\Invalid</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1018,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z982"/>
+  <dimension ref="A1:Z984"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -1106,104 +1118,109 @@
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>199</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>48</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
-        <v>179</v>
+        <v>200</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>180</v>
+        <v>202</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="B11" s="2"/>
+      <c r="A11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
-        <v>57</v>
+        <v>179</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>52</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A13" t="s">
-        <v>58</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>51</v>
-      </c>
+      <c r="B13" s="2"/>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>182</v>
+        <v>59</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>181</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.25" customHeight="1">
       <c r="A17" t="s">
-        <v>194</v>
+        <v>60</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>196</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>194</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>56</v>
+        <v>196</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>62</v>
+        <v>195</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>50</v>
+        <v>197</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B21" s="2"/>
+      <c r="A21" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
@@ -1211,59 +1228,68 @@
     </row>
     <row r="24" spans="1:3" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>183</v>
-      </c>
-      <c r="B24" t="s">
-        <v>184</v>
+        <v>54</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A25" t="s">
-        <v>185</v>
-      </c>
-      <c r="B25" t="s">
-        <v>186</v>
-      </c>
-      <c r="C25" s="2"/>
+      <c r="B25" s="2"/>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
       <c r="A26" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="B26" t="s">
-        <v>193</v>
-      </c>
-      <c r="C26" s="2"/>
+        <v>184</v>
+      </c>
     </row>
     <row r="27" spans="1:3" ht="14.25" customHeight="1">
-      <c r="B27" s="2"/>
+      <c r="A27" t="s">
+        <v>185</v>
+      </c>
+      <c r="B27" t="s">
+        <v>186</v>
+      </c>
+      <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:3" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>187</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>198</v>
-      </c>
+        <v>192</v>
+      </c>
+      <c r="B28" t="s">
+        <v>193</v>
+      </c>
+      <c r="C28" s="2"/>
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A29" t="s">
-        <v>188</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>189</v>
-      </c>
+      <c r="B29" s="2"/>
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" t="s">
+        <v>187</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A31" t="s">
+        <v>188</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A32" t="s">
         <v>190</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B32" s="2" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="32" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>
@@ -2214,6 +2240,8 @@
     <row r="980" ht="14.25" customHeight="1"/>
     <row r="981" ht="14.25" customHeight="1"/>
     <row r="982" ht="14.25" customHeight="1"/>
+    <row r="983" ht="14.25" customHeight="1"/>
+    <row r="984" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>